<commit_message>
Re-protect Excel templates: unlock data cells, keep headers locked
Existing filled templates had every data cell locked (paste from an
external source overwrites the destination cell's style, including
lock state). Re-ran generate_excel_templates.py --protect-existing to
restore column-level unlock on data rows while keeping headers
protected, so cut/paste/move works within data and stays blocked in
headers. No cell values changed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/api/data/excel_templates/degrees.xlsx
+++ b/apps/api/data/excel_templates/degrees.xlsx
@@ -57,7 +57,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
@@ -70,6 +70,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -491,3004 +494,3204 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Master in Philosophy and English Literature</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>DEG-000001</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Literature &amp; Philosophy</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="E2" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Focuses on literary and philosophical texts. Develops analytical and interpretive skills. Studies cultural theory. Emphasises critical reading. Prepares for academic careers.</t>
         </is>
       </c>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="6" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Master in Philosophy and Mathematics</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>DEG-000002</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Mathematical Philosophy</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" t="inlineStr">
+      <c r="E3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Focuses on logic and mathematical reasoning. Develops analytical and abstract thinking. Studies formal systems. Emphasises theoretical inquiry. Prepares for research careers.</t>
         </is>
       </c>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Master in Philosophy and Public Policy</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>DEG-000003</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Policy Studies</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" t="inlineStr">
+      <c r="E4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Focuses on ethical foundations of policy-making. Develops analytical and governance skills. Studies public systems. Emphasises decision frameworks. Prepares for policy roles.</t>
         </is>
       </c>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Master in Philosophy and Religion</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>DEG-000004</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Religious Studies</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" t="inlineStr">
+      <c r="E5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Focuses on philosophical analysis of religion. Develops interpretive and critical skills. Studies belief systems. Emphasises theological inquiry. Prepares for academic roles.</t>
         </is>
       </c>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Master in Photonics</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>DEG-000005</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Physics &amp; Engineering</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F6" t="inlineStr">
+      <c r="E6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Focuses on light manipulation and optical systems. Develops experimental and theoretical skills. Studies wave optics. Emphasises applied physics. Prepares for research roles.</t>
         </is>
       </c>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Master in Photonics and Quantum Sciences</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>DEG-000006</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Quantum Technology</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F7" t="inlineStr">
+      <c r="E7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Focuses on quantum optics and photonics. Develops theoretical and experimental skills. Studies quantum systems. Emphasises advanced research. Prepares for scientific careers.</t>
         </is>
       </c>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Master in Physical Sciences</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>DEG-000007</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Natural Sciences</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F8" t="inlineStr">
+      <c r="E8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Focuses on physics and related sciences. Develops analytical and experimental skills. Studies matter and energy. Emphasises research methods. Prepares for scientific careers.</t>
         </is>
       </c>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Master in Physical Therapy and Rehabilitation</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>DEG-000008</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Rehabilitation Science</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v>2</v>
-      </c>
-      <c r="F9" t="inlineStr">
+      <c r="E9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Focuses on restoring physical function after injury. Develops therapeutic skills. Studies movement recovery. Emphasises clinical rehabilitation. Prepares for therapy careers.</t>
         </is>
       </c>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Master in Physics and Technology of Nanostructures</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>DEG-000009</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Nanotechnology</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>2</v>
-      </c>
-      <c r="F10" t="inlineStr">
+      <c r="E10" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Focuses on engineered nanoscale structures. Develops experimental and fabrication skills. Studies quantum effects. Emphasises advanced materials. Prepares for research roles.</t>
         </is>
       </c>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Master in Physics and Thermal Physics of Innovative Nuclear Power Installations</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>DEG-000010</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Nuclear Energy</t>
         </is>
       </c>
-      <c r="E11" t="n">
-        <v>2</v>
-      </c>
-      <c r="F11" t="inlineStr">
+      <c r="E11" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Focuses on thermal and reactor physics. Develops modelling and engineering skills. Studies nuclear systems. Emphasises energy innovation. Prepares for nuclear industry roles.</t>
         </is>
       </c>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Master in Physics of Complex Systems and Biophysics</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>DEG-000011</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Biophysics</t>
         </is>
       </c>
-      <c r="E12" t="n">
-        <v>2</v>
-      </c>
-      <c r="F12" t="inlineStr">
+      <c r="E12" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Focuses on complex systems in biology and physics. Develops analytical skills. Studies living systems. Emphasises interdisciplinary research. Prepares for scientific careers.</t>
         </is>
       </c>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Master in Physics with Mathematics</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>DEG-000012</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Mathematical Physics</t>
         </is>
       </c>
-      <c r="E13" t="n">
-        <v>2</v>
-      </c>
-      <c r="F13" t="inlineStr">
+      <c r="E13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Focuses on mathematical methods in physics. Develops modelling and analytical skills. Studies theoretical frameworks. Emphasises problem-solving. Prepares for research roles.</t>
         </is>
       </c>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Master in Physics with Planetary and Space Physics</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>DEG-000013</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Space Physics</t>
         </is>
       </c>
-      <c r="E14" t="n">
-        <v>2</v>
-      </c>
-      <c r="F14" t="inlineStr">
+      <c r="E14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Focuses on planetary systems and space environments. Develops analytical skills. Studies solar and planetary physics. Emphasises space science. Prepares for research careers.</t>
         </is>
       </c>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Master in Planning and Management of Tourism Systems</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>DEG-000014</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Tourism Management</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>2</v>
-      </c>
-      <c r="F15" t="inlineStr">
+      <c r="E15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Focuses on tourism system design and management. Develops planning and business skills. Studies tourism flows. Emphasises sustainability. Prepares for tourism industry roles.</t>
         </is>
       </c>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Master in Plasma Physics, Spectroscopy and Self-Organization</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>DEG-000015</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Applied Physics</t>
         </is>
       </c>
-      <c r="E16" t="n">
-        <v>2</v>
-      </c>
-      <c r="F16" t="inlineStr">
+      <c r="E16" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Focuses on plasma diagnostics and systems behaviour. Develops analytical skills. Studies light-matter interaction. Emphasises advanced research. Prepares for physics careers.</t>
         </is>
       </c>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Master in Play Therapy</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>DEG-000016</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>Psychotherapy</t>
         </is>
       </c>
-      <c r="E17" t="n">
-        <v>2</v>
-      </c>
-      <c r="F17" t="inlineStr">
+      <c r="E17" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>Focuses on therapeutic use of play for children. Develops counselling skills. Studies child psychology. Emphasises emotional development. Prepares for clinical therapy roles.</t>
         </is>
       </c>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Master in Podiatric Surgery</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>DEG-000017</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>Surgical Medicine</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>2</v>
-      </c>
-      <c r="F18" t="inlineStr">
+      <c r="E18" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>Focuses on surgical treatment of foot disorders. Develops clinical and surgical skills. Studies anatomy and pathology. Emphasises operative care. Prepares for surgical roles.</t>
         </is>
       </c>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Master in Portuguese and Business</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>DEG-000018</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>Business Communication</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F19" t="inlineStr">
+      <c r="E19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>Focuses on Portuguese language in business contexts. Develops communication skills. Studies commerce and culture. Emphasises international trade. Prepares for business roles.</t>
         </is>
       </c>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Master in Post-production with Sound Design</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>DEG-000019</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>Media Production</t>
         </is>
       </c>
-      <c r="E20" t="n">
-        <v>2</v>
-      </c>
-      <c r="F20" t="inlineStr">
+      <c r="E20" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>Focuses on audio post-production for media. Develops technical and creative skills. Studies sound design. Emphasises film and media industries. Prepares for production roles.</t>
         </is>
       </c>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Master in Power, Electronic and Telecommunication Engineering</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>DEG-000020</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>Electrical Engineering</t>
         </is>
       </c>
-      <c r="E21" t="n">
-        <v>2</v>
-      </c>
-      <c r="F21" t="inlineStr">
+      <c r="E21" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>Focuses on integrated power and communication systems. Develops technical skills. Studies networks and electronics. Emphasises infrastructure. Prepares for engineering roles.</t>
         </is>
       </c>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>Master in Process Engineering</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>DEG-000021</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>Chemical/Industrial Engineering</t>
         </is>
       </c>
-      <c r="E22" t="n">
-        <v>2</v>
-      </c>
-      <c r="F22" t="inlineStr">
+      <c r="E22" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>Focuses on industrial process design and optimisation. Develops engineering skills. Studies production systems. Emphasises efficiency and safety. Prepares for industry roles.</t>
         </is>
       </c>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Master in Professional Archaeology and Comprehensive Heritage Management</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>DEG-000022</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>Archaeology</t>
         </is>
       </c>
-      <c r="E23" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" t="inlineStr">
+      <c r="E23" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>Focuses on archaeological practice and heritage management. Develops field skills. Studies cultural preservation. Emphasises applied archaeology. Prepares for heritage roles.</t>
         </is>
       </c>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Master in Professional Non-surgical Aesthetic Practice</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>DEG-000023</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>Aesthetic Medicine</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>2</v>
-      </c>
-      <c r="F24" t="inlineStr">
+      <c r="E24" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>Focuses on cosmetic non-surgical treatments. Develops clinical and procedural skills. Studies skin aesthetics. Emphasises patient care. Prepares for aesthetic practice roles.</t>
         </is>
       </c>
+      <c r="G24" s="6" t="n"/>
+      <c r="H24" s="6" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Master in Professional Studies in Education</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>DEG-000024</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E25" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" t="inlineStr">
+      <c r="E25" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>Focuses on advanced teaching and learning practice. Develops pedagogical skills. Studies education systems. Emphasises instructional improvement. Prepares for educator roles.</t>
         </is>
       </c>
+      <c r="G25" s="6" t="n"/>
+      <c r="H25" s="6" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Master in Professional Translation Studies</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>DEG-000025</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>Translation Studies</t>
         </is>
       </c>
-      <c r="E26" t="n">
-        <v>2</v>
-      </c>
-      <c r="F26" t="inlineStr">
+      <c r="E26" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>Focuses on advanced translation theory and practice. Develops language skills. Studies translation techniques. Emphasises accuracy and fluency. Prepares for translator roles.</t>
         </is>
       </c>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="6" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>Master in Prostate Cancer Care</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>DEG-000026</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>Oncology</t>
         </is>
       </c>
-      <c r="E27" t="n">
-        <v>2</v>
-      </c>
-      <c r="F27" t="inlineStr">
+      <c r="E27" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>Focuses on diagnosis and treatment of prostate cancer. Develops clinical skills. Studies oncology care pathways. Emphasises patient management. Prepares for healthcare roles.</t>
         </is>
       </c>
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="6" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>Master in Psychology Conversion</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>DEG-000027</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>Conversion Psychology</t>
         </is>
       </c>
-      <c r="E28" t="n">
-        <v>2</v>
-      </c>
-      <c r="F28" t="inlineStr">
+      <c r="E28" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>Focuses on foundational psychology training. Develops core analytical skills. Studies psychological theory. Emphasises transition into field. Prepares for psychology careers.</t>
         </is>
       </c>
+      <c r="G28" s="6" t="n"/>
+      <c r="H28" s="6" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>Master in Psycho-oncology and Palliative Care</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>DEG-000028</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>Health Psychology</t>
         </is>
       </c>
-      <c r="E29" t="n">
-        <v>2</v>
-      </c>
-      <c r="F29" t="inlineStr">
+      <c r="E29" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>Focuses on psychological support in cancer care. Develops clinical intervention skills. Studies patient wellbeing. Emphasises end-of-life care. Prepares for healthcare roles.</t>
         </is>
       </c>
+      <c r="G29" s="6" t="n"/>
+      <c r="H29" s="6" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Master in Public Health, Public Health Nutrition and Epidemiology</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>DEG-000029</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>Public Health Nutrition</t>
         </is>
       </c>
-      <c r="E30" t="n">
-        <v>2</v>
-      </c>
-      <c r="F30" t="inlineStr">
+      <c r="E30" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>Focuses on nutrition and disease prevention. Develops epidemiological skills. Studies diet and population health. Emphasises prevention strategies. Prepares for health roles.</t>
         </is>
       </c>
+      <c r="G30" s="6" t="n"/>
+      <c r="H30" s="6" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Design in Visual Communication and BA in International Studies</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>DEG-000030</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>Design / Communication</t>
         </is>
       </c>
-      <c r="E31" t="n">
+      <c r="E31" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>Combines visual communication with global studies. Covers branding and media. Develops creative skills. Prepares for design careers.</t>
         </is>
       </c>
+      <c r="G31" s="6" t="n"/>
+      <c r="H31" s="6" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Teaching and BA in Mathematics</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>DEG-000031</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>Education / Mathematics</t>
         </is>
       </c>
-      <c r="E32" t="n">
+      <c r="E32" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>Combines teaching with mathematics. Covers pedagogy and quantitative skills. Develops instructional ability. Prepares for teaching roles.</t>
         </is>
       </c>
+      <c r="G32" s="6" t="n"/>
+      <c r="H32" s="6" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Health Science in Traditional Chinese Medicine and BA in International Studies</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>DEG-000032</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>Health / Traditional Medicine</t>
         </is>
       </c>
-      <c r="E33" t="n">
+      <c r="E33" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <t>Combines Chinese medicine with global studies. Covers holistic health systems. Develops clinical knowledge. Prepares for healthcare roles.</t>
         </is>
       </c>
+      <c r="G33" s="6" t="n"/>
+      <c r="H33" s="6" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Teaching and BA in Visual Arts</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>DEG-000033</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>Education / Arts</t>
         </is>
       </c>
-      <c r="E34" t="n">
+      <c r="E34" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>Combines teaching with visual arts practice. Covers pedagogy and creativity. Develops instructional skills. Prepares for arts education roles.</t>
         </is>
       </c>
+      <c r="G34" s="6" t="n"/>
+      <c r="H34" s="6" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Education and BA in International Studies</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>DEG-000034</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E35" t="n">
+      <c r="E35" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
         <is>
           <t>Combines teaching qualifications with global studies. Covers pedagogy and culture. Develops instructional skills. Prepares for education roles.</t>
         </is>
       </c>
+      <c r="G35" s="6" t="n"/>
+      <c r="H35" s="6" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Teaching and BA in Technology</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>DEG-000035</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>Education / Technology</t>
         </is>
       </c>
-      <c r="E36" t="n">
+      <c r="E36" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="6" t="inlineStr">
         <is>
           <t>Combines teaching with technology studies. Covers digital tools and pedagogy. Develops instructional skills. Prepares for STEM education roles.</t>
         </is>
       </c>
+      <c r="G36" s="6" t="n"/>
+      <c r="H36" s="6" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Journalism and Professional Writing and BA in Creative Writing and Literature</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>DEG-000036</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>Journalism / Writing</t>
         </is>
       </c>
-      <c r="E37" t="n">
+      <c r="E37" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
         <is>
           <t>Combines journalism with creative writing. Covers reporting, storytelling, and media. Develops communication skills. Prepares for media careers.</t>
         </is>
       </c>
+      <c r="G37" s="6" t="n"/>
+      <c r="H37" s="6" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Commerce, BA in Psychology</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>DEG-000037</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>Business / Psychology</t>
         </is>
       </c>
-      <c r="E38" t="n">
+      <c r="E38" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>Combines commerce with psychology studies. Covers business strategy and human behaviour. Develops analytical skills. Prepares for corporate roles.</t>
         </is>
       </c>
+      <c r="G38" s="6" t="n"/>
+      <c r="H38" s="6" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Nursing and BA in International Studies</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>DEG-000038</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>Nursing</t>
         </is>
       </c>
-      <c r="E39" t="n">
+      <c r="E39" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>Combines nursing practice with global studies. Covers healthcare systems and patient care. Develops clinical skills. Prepares for nursing careers.</t>
         </is>
       </c>
+      <c r="G39" s="6" t="n"/>
+      <c r="H39" s="6" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Teaching and BA in Humanities</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>DEG-000039</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E40" t="n">
+      <c r="E40" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>Combines teaching qualification with humanities studies. Covers pedagogy and culture. Develops instructional skills. Prepares for education roles.</t>
         </is>
       </c>
+      <c r="G40" s="6" t="n"/>
+      <c r="H40" s="6" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Design in Interior Architecture and BA in International Studies</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>DEG-000040</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>Design / Architecture</t>
         </is>
       </c>
-      <c r="E41" t="n">
+      <c r="E41" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="6" t="inlineStr">
         <is>
           <t>Combines interior design with global studies. Covers spatial design and culture. Develops creative and technical skills. Prepares for design careers.</t>
         </is>
       </c>
+      <c r="G41" s="6" t="n"/>
+      <c r="H41" s="6" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Design in Product Design and BA in International Studies</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>DEG-000041</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>Design / Product</t>
         </is>
       </c>
-      <c r="E42" t="n">
+      <c r="E42" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <t>Combines product design with global studies. Covers innovation and user-centred design. Develops technical skills. Prepares for design industry roles.</t>
         </is>
       </c>
+      <c r="G42" s="6" t="n"/>
+      <c r="H42" s="6" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Medical Science and BA in International Studies</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>DEG-000042</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>Medical Science</t>
         </is>
       </c>
-      <c r="E43" t="n">
+      <c r="E43" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="6" t="inlineStr">
         <is>
           <t>Combines medical science with global studies. Covers biology, health systems, and policy. Develops scientific skills. Prepares for health sector roles.</t>
         </is>
       </c>
+      <c r="G43" s="6" t="n"/>
+      <c r="H43" s="6" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Design in Animation and BA in International Studies</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>DEG-000043</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>Design / International Studies</t>
         </is>
       </c>
-      <c r="E44" t="n">
+      <c r="E44" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="6" t="inlineStr">
         <is>
           <t>Combines animation with global cultural studies. Covers storytelling and media production. Develops creative skills. Prepares for animation and media roles.</t>
         </is>
       </c>
+      <c r="G44" s="6" t="n"/>
+      <c r="H44" s="6" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Design in Photography and BA in International Studies</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>DEG-000044</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>Design / Photography</t>
         </is>
       </c>
-      <c r="E45" t="n">
+      <c r="E45" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <t>Combines photography with international studies. Covers visual storytelling and culture. Develops artistic skills. Prepares for media and photography roles.</t>
         </is>
       </c>
+      <c r="G45" s="6" t="n"/>
+      <c r="H45" s="6" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Commerce and BA in Psychology and Economics</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>DEG-000045</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>Business / Social Science</t>
         </is>
       </c>
-      <c r="E46" t="n">
+      <c r="E46" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="6" t="inlineStr">
         <is>
           <t>Integrates commerce, psychology, and economics. Covers markets, behaviour, and policy. Develops analytical skills. Prepares for finance and consulting roles.</t>
         </is>
       </c>
+      <c r="G46" s="6" t="n"/>
+      <c r="H46" s="6" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Communication in Creative Writing and BA in International Studies</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>DEG-000046</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>Communication / International Studies</t>
         </is>
       </c>
-      <c r="E47" t="n">
+      <c r="E47" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="6" t="inlineStr">
         <is>
           <t>Combines creative writing with global studies. Covers media, culture, and communication. Develops storytelling skills. Prepares for media and international roles.</t>
         </is>
       </c>
+      <c r="G47" s="6" t="n"/>
+      <c r="H47" s="6" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Construction Project Management, BA in International Studies</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>DEG-000047</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
         <is>
           <t>Construction / International Studies</t>
         </is>
       </c>
-      <c r="E48" t="n">
+      <c r="E48" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="6" t="inlineStr">
         <is>
           <t>Combines construction management with global studies. Covers planning, infrastructure, and policy. Develops leadership skills. Prepares for project management roles.</t>
         </is>
       </c>
+      <c r="G48" s="6" t="n"/>
+      <c r="H48" s="6" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Commerce and BA in Psychology</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>DEG-000048</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>Business / Psychology</t>
         </is>
       </c>
-      <c r="E49" t="n">
+      <c r="E49" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F49" s="6" t="inlineStr">
         <is>
           <t>Combines business commerce with psychological science. Covers markets, behaviour, and analytics. Develops interdisciplinary skills. Prepares for business and HR roles.</t>
         </is>
       </c>
+      <c r="G49" s="6" t="n"/>
+      <c r="H49" s="6" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>Bachelor in Transfer Degree</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t>DEG-000049</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t>General Studies</t>
         </is>
       </c>
-      <c r="E50" t="n">
+      <c r="E50" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F50" s="6" t="inlineStr">
         <is>
           <t>Provides foundational academic coursework for transfer. Develops core academic skills. Focuses on university progression pathways. Prepares students for advanced degrees.</t>
         </is>
       </c>
+      <c r="G50" s="6" t="n"/>
+      <c r="H50" s="6" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="6" t="inlineStr">
         <is>
           <t>Bachelor and MBA in Supply Chain Management</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t>DEG-000050</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>Business / Logistics</t>
         </is>
       </c>
-      <c r="E51" t="n">
+      <c r="E51" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F51" s="6" t="inlineStr">
         <is>
           <t>Integrated program covering supply chain and advanced business management. Covers logistics, operations, and strategy. Develops leadership skills. Prepares for senior management roles.</t>
         </is>
       </c>
+      <c r="G51" s="6" t="n"/>
+      <c r="H51" s="6" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Law with English Language Studies</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="6" t="inlineStr">
         <is>
           <t>DEG-000051</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>English Studies</t>
         </is>
       </c>
-      <c r="E52" t="n">
+      <c r="E52" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F52" s="6" t="inlineStr">
         <is>
           <t>Combines law with advanced study of English linguistics and usage. Builds strong written and verbal reasoning. Prepares for careers in law, media, publishing, or public administration.</t>
         </is>
       </c>
+      <c r="G52" s="6" t="n"/>
+      <c r="H52" s="6" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Law with English</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>DEG-000052</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="E53" t="n">
+      <c r="E53" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <t>Combines law with English language and literature studies. Strengthens critical thinking, analysis, and communication. Prepares for careers in law, publishing, education, or media industries.</t>
         </is>
       </c>
+      <c r="G53" s="6" t="n"/>
+      <c r="H53" s="6" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Law with Classical Studies</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>DEG-000053</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>Classical Studies</t>
         </is>
       </c>
-      <c r="E54" t="n">
+      <c r="E54" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F54" s="6" t="inlineStr">
         <is>
           <t>Integrates law with ancient Greek and Roman civilizations. Develops analytical and historical interpretation skills. Prepares for careers in law, academia, heritage, or cultural policy sectors.</t>
         </is>
       </c>
+      <c r="G54" s="6" t="n"/>
+      <c r="H54" s="6" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Law with Criminology</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>DEG-000054</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>Criminology</t>
         </is>
       </c>
-      <c r="E55" t="n">
+      <c r="E55" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <t>Combines law with the study of crime, justice, and society. Develops understanding of criminal behavior and legal responses. Leads to careers in policing, legal practice, or criminal justice policy.</t>
         </is>
       </c>
+      <c r="G55" s="6" t="n"/>
+      <c r="H55" s="6" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Forestry Transfer</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="6" t="inlineStr">
         <is>
           <t>DEG-000055</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>Forestry (Transfer Program)</t>
         </is>
       </c>
-      <c r="E56" t="n">
+      <c r="E56" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F56" s="6" t="inlineStr">
         <is>
           <t>Provides foundational forestry education for academic transfer pathways. Develops basic ecological and scientific skills. Prepares students for advanced forestry studies. Strengthens academic readiness. Supports progression into specialized forestry degrees.</t>
         </is>
       </c>
+      <c r="G56" s="6" t="n"/>
+      <c r="H56" s="6" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Language and Literature Education</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>DEG-000056</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>Education &amp; Language</t>
         </is>
       </c>
-      <c r="E57" t="n">
+      <c r="E57" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F57" s="6" t="inlineStr">
         <is>
           <t>Focuses on teaching languages and literature. Builds pedagogy and communication skills. Graduates work as language teachers.</t>
         </is>
       </c>
+      <c r="G57" s="6" t="n"/>
+      <c r="H57" s="6" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Mathematics with Education</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="6" t="inlineStr">
         <is>
           <t>DEG-000057</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="6" t="inlineStr">
         <is>
           <t>Mathematics Education</t>
         </is>
       </c>
-      <c r="E58" t="n">
+      <c r="E58" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F58" s="6" t="inlineStr">
         <is>
           <t>Focuses on mathematics teaching and learning methods. Builds pedagogical skills. Graduates work in schools or education roles.</t>
         </is>
       </c>
+      <c r="G58" s="6" t="n"/>
+      <c r="H58" s="6" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Italian and Persian</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>DEG-000058</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>Language Studies</t>
         </is>
       </c>
-      <c r="E59" t="n">
+      <c r="E59" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="F59" s="6" t="inlineStr">
         <is>
           <t>Combines Italian and Persian languages. Builds intercultural communication skills. Graduates work in translation and diplomacy.</t>
         </is>
       </c>
+      <c r="G59" s="6" t="n"/>
+      <c r="H59" s="6" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Medical Studies and Doctor of Medicine</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="6" t="inlineStr">
         <is>
           <t>DEG-000059</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D60" s="6" t="inlineStr">
         <is>
           <t>Medical Pathway</t>
         </is>
       </c>
-      <c r="E60" t="n">
+      <c r="E60" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="F60" s="6" t="inlineStr">
         <is>
           <t>Integrated medical training program. Builds clinical and scientific expertise. Graduates become licensed medical practitioners.</t>
         </is>
       </c>
+      <c r="G60" s="6" t="n"/>
+      <c r="H60" s="6" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="6" t="inlineStr">
         <is>
           <t>Bachelor of History Teaching</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="6" t="inlineStr">
         <is>
           <t>DEG-000060</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61" s="6" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E61" t="n">
+      <c r="E61" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="F61" s="6" t="inlineStr">
         <is>
           <t>Studies methods of teaching history. Develops pedagogical skills. Focuses on classroom instruction. Graduates work as educators.</t>
         </is>
       </c>
+      <c r="G61" s="6" t="n"/>
+      <c r="H61" s="6" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="6" t="inlineStr">
         <is>
           <t>PhD in Fluids Engineering</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="6" t="inlineStr">
         <is>
           <t>DEG-000061</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62" s="6" t="inlineStr">
         <is>
           <t>Mechanical Engineering</t>
         </is>
       </c>
-      <c r="E62" t="n">
+      <c r="E62" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="F62" s="6" t="inlineStr">
         <is>
           <t>Studies fluid flow and engineering system design. Develops expertise in computational modeling and experimental research. Focuses on industrial and energy applications. Graduates work in research, aerospace, and engineering firms.</t>
         </is>
       </c>
+      <c r="G62" s="6" t="n"/>
+      <c r="H62" s="6" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="6" t="inlineStr">
         <is>
           <t>PhD in Food and Biochemical Technology</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="6" t="inlineStr">
         <is>
           <t>DEG-000062</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D63" s="6" t="inlineStr">
         <is>
           <t>Food Science</t>
         </is>
       </c>
-      <c r="E63" t="n">
+      <c r="E63" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F63" s="6" t="inlineStr">
         <is>
           <t>Combines food science with biochemical technologies. Develops expertise in food processing and biochemical research. Focuses on improving food quality and innovation. Graduates work in academia, biotechnology, and food industries.</t>
         </is>
       </c>
+      <c r="G63" s="6" t="n"/>
+      <c r="H63" s="6" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="6" t="inlineStr">
         <is>
           <t>PhD in Food Systems</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="6" t="inlineStr">
         <is>
           <t>DEG-000063</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="6" t="inlineStr">
         <is>
           <t>Food Systems</t>
         </is>
       </c>
-      <c r="E64" t="n">
+      <c r="E64" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F64" s="6" t="inlineStr">
         <is>
           <t>Explores food production, distribution, and consumption systems. Develops interdisciplinary research and policy skills. Focuses on sustainability and resilience. Graduates work in academia, government, and nonprofit organizations.</t>
         </is>
       </c>
+      <c r="G64" s="6" t="n"/>
+      <c r="H64" s="6" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="6" t="inlineStr">
         <is>
           <t>PhD in Gender Studies</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="6" t="inlineStr">
         <is>
           <t>DEG-000064</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65" s="6" t="inlineStr">
         <is>
           <t>Gender Studies</t>
         </is>
       </c>
-      <c r="E65" t="n">
+      <c r="E65" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F65" s="6" t="inlineStr">
         <is>
           <t>Explores gender through social, political, and cultural research. Develops critical thinking and interdisciplinary research skills. Focuses on identity and equality. Graduates work in academia, policy, and community organizations.</t>
         </is>
       </c>
+      <c r="G65" s="6" t="n"/>
+      <c r="H65" s="6" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="6" t="inlineStr">
         <is>
           <t>PhD in Geodesy and Geoinformatics</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="6" t="inlineStr">
         <is>
           <t>DEG-000065</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D66" s="6" t="inlineStr">
         <is>
           <t>Geospatial Science</t>
         </is>
       </c>
-      <c r="E66" t="n">
+      <c r="E66" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F66" s="6" t="inlineStr">
         <is>
           <t>Combines geodesy with digital geographic information systems. Develops expertise in spatial analysis and geospatial technologies. Focuses on Earth measurement and mapping. Graduates work in academia, surveying, and GIS industries.</t>
         </is>
       </c>
+      <c r="G66" s="6" t="n"/>
+      <c r="H66" s="6" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="6" t="inlineStr">
         <is>
           <t>PhD in Geography and Earth Science</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B67" s="6" t="inlineStr">
         <is>
           <t>DEG-000066</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D67" s="6" t="inlineStr">
         <is>
           <t>Earth Science</t>
         </is>
       </c>
-      <c r="E67" t="n">
+      <c r="E67" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="F67" s="6" t="inlineStr">
         <is>
           <t>Combines geography with Earth science research. Develops expertise in environmental systems and geospatial analysis. Focuses on understanding Earth's processes. Graduates work in academia, environmental consulting, and government.</t>
         </is>
       </c>
+      <c r="G67" s="6" t="n"/>
+      <c r="H67" s="6" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="6" t="inlineStr">
         <is>
           <t>PhD in Geometry and Topology</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B68" s="6" t="inlineStr">
         <is>
           <t>DEG-000067</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr">
+      <c r="D68" s="6" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="E68" t="n">
+      <c r="E68" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="F68" s="6" t="inlineStr">
         <is>
           <t>Studies the properties and structures of geometric spaces. Develops expertise in abstract mathematics and theoretical research. Focuses on advanced mathematical concepts. Graduates work in academia, research, and higher education.</t>
         </is>
       </c>
+      <c r="G68" s="6" t="n"/>
+      <c r="H68" s="6" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="6" t="inlineStr">
         <is>
           <t>PhD in Geospatial Analytics</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="6" t="inlineStr">
         <is>
           <t>DEG-000068</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D69" s="6" t="inlineStr">
         <is>
           <t>Data Science</t>
         </is>
       </c>
-      <c r="E69" t="n">
+      <c r="E69" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F69" s="6" t="inlineStr">
         <is>
           <t>Studies advanced analysis of geographic and spatial data. Develops expertise in GIS, machine learning, and predictive modeling. Focuses on spatial decision-making. Graduates work in academia, government, and technology industries.</t>
         </is>
       </c>
+      <c r="G69" s="6" t="n"/>
+      <c r="H69" s="6" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="6" t="inlineStr">
         <is>
           <t>PhD in Grain Science</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B70" s="6" t="inlineStr">
         <is>
           <t>DEG-000069</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C70" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D70" s="6" t="inlineStr">
         <is>
           <t>Agricultural Science</t>
         </is>
       </c>
-      <c r="E70" t="n">
+      <c r="E70" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="F70" s="6" t="inlineStr">
         <is>
           <t>Studies grain production, processing, and quality. Develops expertise in cereal chemistry and agricultural research. Focuses on food quality and sustainable production. Graduates work in academia, agriculture, and food industries.</t>
         </is>
       </c>
+      <c r="G70" s="6" t="n"/>
+      <c r="H70" s="6" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
+      <c r="A71" s="6" t="inlineStr">
         <is>
           <t>PhD in Health Economics and Policy</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B71" s="6" t="inlineStr">
         <is>
           <t>DEG-000070</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C71" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr">
+      <c r="D71" s="6" t="inlineStr">
         <is>
           <t>Health Economics</t>
         </is>
       </c>
-      <c r="E71" t="n">
+      <c r="E71" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="F71" s="6" t="inlineStr">
         <is>
           <t>Integrates economic analysis with healthcare policy research. Develops expertise in health financing and policy evaluation. Focuses on improving health systems. Graduates work in academia, government, and healthcare organizations.</t>
         </is>
       </c>
+      <c r="G71" s="6" t="n"/>
+      <c r="H71" s="6" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
+      <c r="A72" s="6" t="inlineStr">
         <is>
           <t>PhD in Hispanic Studies and Comparative Literature</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B72" s="6" t="inlineStr">
         <is>
           <t>DEG-000071</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C72" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D72" s="6" t="inlineStr">
         <is>
           <t>Literature</t>
         </is>
       </c>
-      <c r="E72" t="n">
+      <c r="E72" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F72" s="6" t="inlineStr">
         <is>
           <t>Combines Hispanic studies with comparative literary research. Develops expertise in literary analysis and cross-cultural interpretation. Focuses on global literary traditions. Graduates work in academia, publishing, and education.</t>
         </is>
       </c>
+      <c r="G72" s="6" t="n"/>
+      <c r="H72" s="6" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
+      <c r="A73" s="6" t="inlineStr">
         <is>
           <t>PhD in History of Art and Archaeology</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B73" s="6" t="inlineStr">
         <is>
           <t>DEG-000072</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C73" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D73" s="6" t="inlineStr">
         <is>
           <t>Art History</t>
         </is>
       </c>
-      <c r="E73" t="n">
+      <c r="E73" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F73" s="6" t="inlineStr">
         <is>
           <t>Combines art history with archaeological research. Develops expertise in material culture and historical interpretation. Focuses on ancient and historical artifacts. Graduates work in academia, museums, and heritage organizations.</t>
         </is>
       </c>
+      <c r="G73" s="6" t="n"/>
+      <c r="H73" s="6" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="A74" s="6" t="inlineStr">
         <is>
           <t>PhD in Laser, Photonics and Vision</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B74" s="6" t="inlineStr">
         <is>
           <t>DEG-000073</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C74" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D74" s="6" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="E74" t="n">
+      <c r="E74" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="F74" s="6" t="inlineStr">
         <is>
           <t>Studies laser systems, photonics, and optical vision technologies. Develops expertise in optics, imaging, and applied physics. Focuses on light-based technologies. Graduates work in academia, research labs, and optical industries.</t>
         </is>
       </c>
+      <c r="G74" s="6" t="n"/>
+      <c r="H74" s="6" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="6" t="inlineStr">
         <is>
           <t>PhD in Latin American Cultural Studies</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="6" t="inlineStr">
         <is>
           <t>DEG-000074</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D75" s="6" t="inlineStr">
         <is>
           <t>Cultural Studies</t>
         </is>
       </c>
-      <c r="E75" t="n">
+      <c r="E75" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F75" s="6" t="inlineStr">
         <is>
           <t>Explores cultural production, identity, and history in Latin America. Develops expertise in literary and cultural theory. Focuses on regional cultural expression. Graduates work in academia, publishing, and cultural organizations.</t>
         </is>
       </c>
+      <c r="G75" s="6" t="n"/>
+      <c r="H75" s="6" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" s="6" t="inlineStr">
         <is>
           <t>PhD in Leadership and Policy Studies in Education</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="6" t="inlineStr">
         <is>
           <t>DEG-000075</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C76" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D76" s="6" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E76" t="n">
+      <c r="E76" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F76" s="6" t="inlineStr">
         <is>
           <t>Examines leadership and policy in educational systems. Develops expertise in administration, policy analysis, and school leadership. Focuses on educational improvement. Graduates work in academia, schools, and government agencies.</t>
         </is>
       </c>
+      <c r="G76" s="6" t="n"/>
+      <c r="H76" s="6" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
+      <c r="A77" s="6" t="inlineStr">
         <is>
           <t>PhD in Management Finance</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B77" s="6" t="inlineStr">
         <is>
           <t>DEG-000076</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C77" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D77" s="6" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="E77" t="n">
+      <c r="E77" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F77" t="inlineStr">
+      <c r="F77" s="6" t="inlineStr">
         <is>
           <t>Integrates financial management with organizational strategy. Develops expertise in corporate finance, investment, and risk management. Focuses on financial decision-making. Graduates work in finance, corporations, and consulting.</t>
         </is>
       </c>
+      <c r="G77" s="6" t="n"/>
+      <c r="H77" s="6" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
+      <c r="A78" s="6" t="inlineStr">
         <is>
           <t>PhD in Marine Engine Engineering</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="B78" s="6" t="inlineStr">
         <is>
           <t>DEG-000077</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C78" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="D78" s="6" t="inlineStr">
         <is>
           <t>Marine Engineering</t>
         </is>
       </c>
-      <c r="E78" t="n">
+      <c r="E78" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F78" t="inlineStr">
+      <c r="F78" s="6" t="inlineStr">
         <is>
           <t>Focuses on design and maintenance of marine propulsion systems. Develops expertise in mechanical and marine systems engineering. Focuses on ship engine performance. Graduates work in shipping, engineering, and maritime industries.</t>
         </is>
       </c>
+      <c r="G78" s="6" t="n"/>
+      <c r="H78" s="6" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
+      <c r="A79" s="6" t="inlineStr">
         <is>
           <t>PhD in Marketing and Entrepreneurship</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B79" s="6" t="inlineStr">
         <is>
           <t>DEG-000078</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C79" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D79" s="6" t="inlineStr">
         <is>
           <t>Entrepreneurship</t>
         </is>
       </c>
-      <c r="E79" t="n">
+      <c r="E79" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F79" t="inlineStr">
+      <c r="F79" s="6" t="inlineStr">
         <is>
           <t>Studies marketing strategies for new ventures and startups. Develops expertise in innovation, branding, and business development. Focuses on entrepreneurial growth. Graduates work in startups, consulting, and business development.</t>
         </is>
       </c>
+      <c r="G79" s="6" t="n"/>
+      <c r="H79" s="6" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
+      <c r="A80" s="6" t="inlineStr">
         <is>
           <t>PhD in Phonetics and Phonology</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B80" s="6" t="inlineStr">
         <is>
           <t>DEG-000079</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C80" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr">
+      <c r="D80" s="6" t="inlineStr">
         <is>
           <t>Linguistics</t>
         </is>
       </c>
-      <c r="E80" t="n">
+      <c r="E80" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F80" t="inlineStr">
+      <c r="F80" s="6" t="inlineStr">
         <is>
           <t>Combines speech sound analysis with language sound systems. Develops expertise in linguistic theory and speech research. Focuses on sound structure and communication. Graduates work in academia, linguistics, and speech technology.</t>
         </is>
       </c>
+      <c r="G80" s="6" t="n"/>
+      <c r="H80" s="6" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
+      <c r="A81" s="6" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Nursing and Allied Health</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B81" s="6" t="inlineStr">
         <is>
           <t>DEG-000080</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C81" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D81" s="6" t="inlineStr">
         <is>
           <t>Nursing and Allied Health</t>
         </is>
       </c>
-      <c r="E81" t="n">
-        <v>2</v>
-      </c>
-      <c r="F81" t="inlineStr">
+      <c r="E81" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F81" s="6" t="inlineStr">
         <is>
           <t>Studies basic nursing and healthcare support. Develops clinical and patient care skills. Focuses on healthcare services. Prepares graduates for healthcare support roles.</t>
         </is>
       </c>
+      <c r="G81" s="6" t="n"/>
+      <c r="H81" s="6" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
+      <c r="A82" s="6" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Medical Assistant</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B82" s="6" t="inlineStr">
         <is>
           <t>DEG-000081</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C82" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr">
+      <c r="D82" s="6" t="inlineStr">
         <is>
           <t>Medical Assistance</t>
         </is>
       </c>
-      <c r="E82" t="n">
-        <v>2</v>
-      </c>
-      <c r="F82" t="inlineStr">
+      <c r="E82" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F82" s="6" t="inlineStr">
         <is>
           <t>Studies clinical and administrative healthcare support. Develops patient care skills. Focuses on medical office practice. Prepares graduates for healthcare support roles.</t>
         </is>
       </c>
+      <c r="G82" s="6" t="n"/>
+      <c r="H82" s="6" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
+      <c r="A83" s="6" t="inlineStr">
         <is>
           <t>Associate of Science in Radiography</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="B83" s="6" t="inlineStr">
         <is>
           <t>DEG-000082</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C83" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
+      <c r="D83" s="6" t="inlineStr">
         <is>
           <t>Radiography</t>
         </is>
       </c>
-      <c r="E83" t="n">
-        <v>2</v>
-      </c>
-      <c r="F83" t="inlineStr">
+      <c r="E83" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F83" s="6" t="inlineStr">
         <is>
           <t>Studies medical imaging and radiographic techniques. Develops imaging, patient care, and technical skills. Focuses on diagnostic imaging procedures. Graduates work in hospitals and medical imaging departments.</t>
         </is>
       </c>
+      <c r="G83" s="6" t="n"/>
+      <c r="H83" s="6" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
+      <c r="A84" s="6" t="inlineStr">
         <is>
           <t>Associate of Arts in Marketing</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B84" s="6" t="inlineStr">
         <is>
           <t>DEG-000083</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C84" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="D84" s="6" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="E84" t="n">
-        <v>2</v>
-      </c>
-      <c r="F84" t="inlineStr">
+      <c r="E84" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F84" s="6" t="inlineStr">
         <is>
           <t>Studies marketing strategies and consumer behavior. Develops communication, analytical, and promotional skills. Focuses on branding, advertising, and market research. Graduates work in marketing, sales, and retail.</t>
         </is>
       </c>
+      <c r="G84" s="6" t="n"/>
+      <c r="H84" s="6" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
+      <c r="A85" s="6" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Dental Hygiene</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B85" s="6" t="inlineStr">
         <is>
           <t>DEG-000084</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C85" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D85" s="6" t="inlineStr">
         <is>
           <t>Dental Hygiene</t>
         </is>
       </c>
-      <c r="E85" t="n">
-        <v>2</v>
-      </c>
-      <c r="F85" t="inlineStr">
+      <c r="E85" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" s="6" t="inlineStr">
         <is>
           <t>Studies preventive dental care and oral health. Develops clinical, patient care, and communication skills. Focuses on dental hygiene procedures and education. Graduates work in dental clinics and healthcare facilities.</t>
         </is>
       </c>
+      <c r="G85" s="6" t="n"/>
+      <c r="H85" s="6" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
+      <c r="A86" s="6" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Radiography</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B86" s="6" t="inlineStr">
         <is>
           <t>DEG-000085</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C86" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D86" s="6" t="inlineStr">
         <is>
           <t>Radiography</t>
         </is>
       </c>
-      <c r="E86" t="n">
-        <v>2</v>
-      </c>
-      <c r="F86" t="inlineStr">
+      <c r="E86" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F86" s="6" t="inlineStr">
         <is>
           <t>Studies diagnostic imaging and radiographic procedures. Develops imaging, patient care, and technical skills. Focuses on producing medical images for diagnosis. Graduates work in hospitals and diagnostic imaging centers.</t>
         </is>
       </c>
+      <c r="G86" s="6" t="n"/>
+      <c r="H86" s="6" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
+      <c r="A87" s="6" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Diagnostic Medical Sonography</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B87" s="6" t="inlineStr">
         <is>
           <t>DEG-000086</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C87" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D87" s="6" t="inlineStr">
         <is>
           <t>Diagnostic Medical Sonography</t>
         </is>
       </c>
-      <c r="E87" t="n">
-        <v>2</v>
-      </c>
-      <c r="F87" t="inlineStr">
+      <c r="E87" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F87" s="6" t="inlineStr">
         <is>
           <t>Studies ultrasound imaging and patient care. Develops diagnostic imaging, technical, and clinical skills. Focuses on safe and accurate medical sonography. Prepares graduates for careers as diagnostic medical sonographers.</t>
         </is>
       </c>
+      <c r="G87" s="6" t="n"/>
+      <c r="H87" s="6" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr">
+      <c r="A88" s="6" t="inlineStr">
         <is>
           <t>Associate of Science in Music Production</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B88" s="6" t="inlineStr">
         <is>
           <t>DEG-000087</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="C88" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="D88" s="6" t="inlineStr">
         <is>
           <t>Music Production</t>
         </is>
       </c>
-      <c r="E88" t="n">
-        <v>2</v>
-      </c>
-      <c r="F88" t="inlineStr">
+      <c r="E88" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F88" s="6" t="inlineStr">
         <is>
           <t>Studies audio recording, music technology, and production. Develops recording, editing, and sound design skills. Focuses on creating professional music productions. Graduates work in recording studios and media production.</t>
         </is>
       </c>
+      <c r="G88" s="6" t="n"/>
+      <c r="H88" s="6" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr">
+      <c r="A89" s="6" t="inlineStr">
         <is>
           <t>Associate of Applied Science</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B89" s="6" t="inlineStr">
         <is>
           <t>DEG-000088</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C89" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="D89" s="6" t="inlineStr">
         <is>
           <t>Applied Science</t>
         </is>
       </c>
-      <c r="E89" t="n">
-        <v>2</v>
-      </c>
-      <c r="F89" t="inlineStr">
+      <c r="E89" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F89" s="6" t="inlineStr">
         <is>
           <t>Studies practical scientific and technical applications. Develops laboratory, technical, and problem-solving skills. Focuses on career-ready scientific knowledge. Graduates work in technical, healthcare, and industrial roles.</t>
         </is>
       </c>
+      <c r="G89" s="6" t="n"/>
+      <c r="H89" s="6" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr">
+      <c r="A90" s="6" t="inlineStr">
         <is>
           <t>Associate of Science in Nursing</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B90" s="6" t="inlineStr">
         <is>
           <t>DEG-000089</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C90" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr">
+      <c r="D90" s="6" t="inlineStr">
         <is>
           <t>Nursing</t>
         </is>
       </c>
-      <c r="E90" t="n">
-        <v>2</v>
-      </c>
-      <c r="F90" t="inlineStr">
+      <c r="E90" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F90" s="6" t="inlineStr">
         <is>
           <t>Studies nursing science and patient-centered care. Develops clinical, communication, and healthcare skills. Focuses on safe nursing practice and health promotion. Graduates work in hospitals, clinics, and healthcare facilities.</t>
         </is>
       </c>
+      <c r="G90" s="6" t="n"/>
+      <c r="H90" s="6" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr">
+      <c r="A91" s="6" t="inlineStr">
         <is>
           <t>Associate of Arts</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B91" s="6" t="inlineStr">
         <is>
           <t>DEG-000090</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C91" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr">
+      <c r="D91" s="6" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="E91" t="n">
-        <v>2</v>
-      </c>
-      <c r="F91" t="inlineStr">
+      <c r="E91" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F91" s="6" t="inlineStr">
         <is>
           <t>Studies humanities, social sciences, and communication. Develops critical thinking, writing, and analytical skills. Focuses on broad academic preparation. Graduates continue higher education or enter diverse professional fields.</t>
         </is>
       </c>
+      <c r="G91" s="6" t="n"/>
+      <c r="H91" s="6" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
+      <c r="A92" s="6" t="inlineStr">
         <is>
           <t>Associate of Arts Degree</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
+      <c r="B92" s="6" t="inlineStr">
         <is>
           <t>DEG-000091</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
+      <c r="C92" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr">
+      <c r="D92" s="6" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="E92" t="n">
-        <v>2</v>
-      </c>
-      <c r="F92" t="inlineStr">
+      <c r="E92" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F92" s="6" t="inlineStr">
         <is>
           <t>Studies a broad range of humanities and social sciences. Develops communication, research, and critical thinking skills. Focuses on transferable academic knowledge. Graduates continue higher education or pursue entry-level careers.</t>
         </is>
       </c>
+      <c r="G92" s="6" t="n"/>
+      <c r="H92" s="6" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr">
+      <c r="A93" s="6" t="inlineStr">
         <is>
           <t>Associate of Nursing</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B93" s="6" t="inlineStr">
         <is>
           <t>DEG-000092</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C93" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr">
+      <c r="D93" s="6" t="inlineStr">
         <is>
           <t>Nursing</t>
         </is>
       </c>
-      <c r="E93" t="n">
-        <v>2</v>
-      </c>
-      <c r="F93" t="inlineStr">
+      <c r="E93" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F93" s="6" t="inlineStr">
         <is>
           <t>Studies patient care and foundational nursing practice. Develops clinical, communication, and healthcare skills. Focuses on evidence-based nursing and patient safety. Graduates work in hospitals, clinics, and healthcare facilities.</t>
         </is>
       </c>
+      <c r="G93" s="6" t="n"/>
+      <c r="H93" s="6" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr">
+      <c r="A94" s="6" t="inlineStr">
         <is>
           <t>Associate of Science in Business</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B94" s="6" t="inlineStr">
         <is>
           <t>DEG-000093</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
+      <c r="C94" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr">
+      <c r="D94" s="6" t="inlineStr">
         <is>
           <t>Business</t>
         </is>
       </c>
-      <c r="E94" t="n">
-        <v>2</v>
-      </c>
-      <c r="F94" t="inlineStr">
+      <c r="E94" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F94" s="6" t="inlineStr">
         <is>
           <t>Studies core business principles and organizational practices. Develops communication, management, and analytical skills. Focuses on finance, marketing, and operations. Graduates work in business support, retail, and administration.</t>
         </is>
       </c>
+      <c r="G94" s="6" t="n"/>
+      <c r="H94" s="6" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr">
+      <c r="A95" s="6" t="inlineStr">
         <is>
           <t>Associate of Science</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="B95" s="6" t="inlineStr">
         <is>
           <t>DEG-000094</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C95" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr">
+      <c r="D95" s="6" t="inlineStr">
         <is>
           <t>Science</t>
         </is>
       </c>
-      <c r="E95" t="n">
-        <v>2</v>
-      </c>
-      <c r="F95" t="inlineStr">
+      <c r="E95" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F95" s="6" t="inlineStr">
         <is>
           <t>Studies foundational scientific concepts and methods. Develops laboratory, analytical, and problem-solving skills. Focuses on biology, chemistry, and scientific inquiry. Graduates continue science studies or work in technical fields.</t>
         </is>
       </c>
+      <c r="G95" s="6" t="n"/>
+      <c r="H95" s="6" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
+      <c r="A96" s="6" t="inlineStr">
         <is>
           <t>Associate of Science in Business Administration</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B96" s="6" t="inlineStr">
         <is>
           <t>DEG-000095</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C96" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr">
+      <c r="D96" s="6" t="inlineStr">
         <is>
           <t>Business Administration</t>
         </is>
       </c>
-      <c r="E96" t="n">
-        <v>2</v>
-      </c>
-      <c r="F96" t="inlineStr">
+      <c r="E96" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F96" s="6" t="inlineStr">
         <is>
           <t>Studies business operations and management fundamentals. Develops organizational, communication, and leadership skills. Focuses on business strategy and workplace effectiveness. Graduates work in administration, sales, and operations.</t>
         </is>
       </c>
+      <c r="G96" s="6" t="n"/>
+      <c r="H96" s="6" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
+      <c r="A97" s="6" t="inlineStr">
         <is>
           <t>Associate of Science in Biology and Ecology</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="B97" s="6" t="inlineStr">
         <is>
           <t>DEG-000096</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
+      <c r="C97" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr">
+      <c r="D97" s="6" t="inlineStr">
         <is>
           <t>Biology and Ecology</t>
         </is>
       </c>
-      <c r="E97" t="n">
-        <v>2</v>
-      </c>
-      <c r="F97" t="inlineStr">
+      <c r="E97" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F97" s="6" t="inlineStr">
         <is>
           <t>Studies biological systems and ecological processes. Develops laboratory, fieldwork, and analytical skills. Focuses on ecosystems, biodiversity, and environmental science. Graduates work in environmental organizations and laboratories.</t>
         </is>
       </c>
+      <c r="G97" s="6" t="n"/>
+      <c r="H97" s="6" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
+      <c r="A98" s="6" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Accounting</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
+      <c r="B98" s="6" t="inlineStr">
         <is>
           <t>DEG-000097</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
+      <c r="C98" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr">
+      <c r="D98" s="6" t="inlineStr">
         <is>
           <t>Accounting</t>
         </is>
       </c>
-      <c r="E98" t="n">
-        <v>2</v>
-      </c>
-      <c r="F98" t="inlineStr">
+      <c r="E98" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F98" s="6" t="inlineStr">
         <is>
           <t>Studies accounting principles and financial reporting. Develops bookkeeping, financial analysis, and accounting software skills. Focuses on business finance and compliance. Graduates work in accounting, bookkeeping, and finance support.</t>
         </is>
       </c>
+      <c r="G98" s="6" t="n"/>
+      <c r="H98" s="6" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr">
+      <c r="A99" s="6" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Hospitality Management</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="B99" s="6" t="inlineStr">
         <is>
           <t>DEG-000098</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C99" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr">
+      <c r="D99" s="6" t="inlineStr">
         <is>
           <t>Hospitality Management</t>
         </is>
       </c>
-      <c r="E99" t="n">
-        <v>2</v>
-      </c>
-      <c r="F99" t="inlineStr">
+      <c r="E99" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F99" s="6" t="inlineStr">
         <is>
           <t>Studies hospitality operations and customer service management. Develops leadership, communication, and operational skills. Focuses on hotels, tourism, and guest satisfaction. Graduates work in hospitality, tourism, and hotel management.</t>
         </is>
       </c>
+      <c r="G99" s="6" t="n"/>
+      <c r="H99" s="6" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr">
+      <c r="A100" s="6" t="inlineStr">
         <is>
           <t>Associate of Science in Computer Science</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
+      <c r="B100" s="6" t="inlineStr">
         <is>
           <t>DEG-000099</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
+      <c r="C100" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr">
+      <c r="D100" s="6" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="E100" t="n">
-        <v>2</v>
-      </c>
-      <c r="F100" t="inlineStr">
+      <c r="E100" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F100" s="6" t="inlineStr">
         <is>
           <t>Studies computing principles and software development. Develops programming, analytical, and technical problem-solving skills. Focuses on algorithms, databases, and computer systems. Graduates work in IT support and software development.</t>
         </is>
       </c>
+      <c r="G100" s="6" t="n"/>
+      <c r="H100" s="6" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
+      <c r="A101" s="6" t="inlineStr">
         <is>
           <t>Associate of Arts in Business Administration</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
+      <c r="B101" s="6" t="inlineStr">
         <is>
           <t>DEG-000100</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
+      <c r="C101" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr">
+      <c r="D101" s="6" t="inlineStr">
         <is>
           <t>Business Administration</t>
         </is>
       </c>
-      <c r="E101" t="n">
-        <v>2</v>
-      </c>
-      <c r="F101" t="inlineStr">
+      <c r="E101" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F101" s="6" t="inlineStr">
         <is>
           <t>Studies business operations and organizational management. Develops leadership, communication, and administrative skills. Focuses on finance, marketing, and business practices. Graduates work in administration, retail, and business support.</t>
         </is>
       </c>
+      <c r="G101" s="6" t="n"/>
+      <c r="H101" s="6" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1" password="DB2D"/>

</xml_diff>

<commit_message>
Regenerate Excel import templates from schema (adds Organization.serial_number)
Reran generate_excel_templates.py --force against the current schema.prisma
so organizations.xlsx picks up the new serial_number column, then pasted
every existing row from the old templates back into the fresh ones (verified
0 cell mismatches across all 9 populated templates).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/api/data/excel_templates/degrees.xlsx
+++ b/apps/api/data/excel_templates/degrees.xlsx
@@ -57,7 +57,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
@@ -70,9 +70,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -494,3204 +491,3004 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Master in Philosophy and English Literature</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>DEG-000001</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Literature &amp; Philosophy</t>
         </is>
       </c>
-      <c r="E2" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>Focuses on literary and philosophical texts. Develops analytical and interpretive skills. Studies cultural theory. Emphasises critical reading. Prepares for academic careers.</t>
         </is>
       </c>
-      <c r="G2" s="6" t="n"/>
-      <c r="H2" s="6" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Master in Philosophy and Mathematics</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>DEG-000002</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Mathematical Philosophy</t>
         </is>
       </c>
-      <c r="E3" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>Focuses on logic and mathematical reasoning. Develops analytical and abstract thinking. Studies formal systems. Emphasises theoretical inquiry. Prepares for research careers.</t>
         </is>
       </c>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Master in Philosophy and Public Policy</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>DEG-000003</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Policy Studies</t>
         </is>
       </c>
-      <c r="E4" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Focuses on ethical foundations of policy-making. Develops analytical and governance skills. Studies public systems. Emphasises decision frameworks. Prepares for policy roles.</t>
         </is>
       </c>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Master in Philosophy and Religion</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>DEG-000004</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Religious Studies</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>Focuses on philosophical analysis of religion. Develops interpretive and critical skills. Studies belief systems. Emphasises theological inquiry. Prepares for academic roles.</t>
         </is>
       </c>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Master in Photonics</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>DEG-000005</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Physics &amp; Engineering</t>
         </is>
       </c>
-      <c r="E6" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>Focuses on light manipulation and optical systems. Develops experimental and theoretical skills. Studies wave optics. Emphasises applied physics. Prepares for research roles.</t>
         </is>
       </c>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Master in Photonics and Quantum Sciences</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>DEG-000006</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Quantum Technology</t>
         </is>
       </c>
-      <c r="E7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="inlineStr">
         <is>
           <t>Focuses on quantum optics and photonics. Develops theoretical and experimental skills. Studies quantum systems. Emphasises advanced research. Prepares for scientific careers.</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Master in Physical Sciences</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>DEG-000007</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Natural Sciences</t>
         </is>
       </c>
-      <c r="E8" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>Focuses on physics and related sciences. Develops analytical and experimental skills. Studies matter and energy. Emphasises research methods. Prepares for scientific careers.</t>
         </is>
       </c>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Master in Physical Therapy and Rehabilitation</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>DEG-000008</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Rehabilitation Science</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>Focuses on restoring physical function after injury. Develops therapeutic skills. Studies movement recovery. Emphasises clinical rehabilitation. Prepares for therapy careers.</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Master in Physics and Technology of Nanostructures</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>DEG-000009</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Nanotechnology</t>
         </is>
       </c>
-      <c r="E10" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="E10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>Focuses on engineered nanoscale structures. Develops experimental and fabrication skills. Studies quantum effects. Emphasises advanced materials. Prepares for research roles.</t>
         </is>
       </c>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Master in Physics and Thermal Physics of Innovative Nuclear Power Installations</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>DEG-000010</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Nuclear Energy</t>
         </is>
       </c>
-      <c r="E11" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="E11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>Focuses on thermal and reactor physics. Develops modelling and engineering skills. Studies nuclear systems. Emphasises energy innovation. Prepares for nuclear industry roles.</t>
         </is>
       </c>
-      <c r="G11" s="6" t="n"/>
-      <c r="H11" s="6" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Master in Physics of Complex Systems and Biophysics</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>DEG-000011</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Biophysics</t>
         </is>
       </c>
-      <c r="E12" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="E12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" t="inlineStr">
         <is>
           <t>Focuses on complex systems in biology and physics. Develops analytical skills. Studies living systems. Emphasises interdisciplinary research. Prepares for scientific careers.</t>
         </is>
       </c>
-      <c r="G12" s="6" t="n"/>
-      <c r="H12" s="6" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Master in Physics with Mathematics</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>DEG-000012</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Mathematical Physics</t>
         </is>
       </c>
-      <c r="E13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="E13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" t="inlineStr">
         <is>
           <t>Focuses on mathematical methods in physics. Develops modelling and analytical skills. Studies theoretical frameworks. Emphasises problem-solving. Prepares for research roles.</t>
         </is>
       </c>
-      <c r="G13" s="6" t="n"/>
-      <c r="H13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Master in Physics with Planetary and Space Physics</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>DEG-000013</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Space Physics</t>
         </is>
       </c>
-      <c r="E14" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="E14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" t="inlineStr">
         <is>
           <t>Focuses on planetary systems and space environments. Develops analytical skills. Studies solar and planetary physics. Emphasises space science. Prepares for research careers.</t>
         </is>
       </c>
-      <c r="G14" s="6" t="n"/>
-      <c r="H14" s="6" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Master in Planning and Management of Tourism Systems</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>DEG-000014</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Tourism Management</t>
         </is>
       </c>
-      <c r="E15" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="E15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" t="inlineStr">
         <is>
           <t>Focuses on tourism system design and management. Develops planning and business skills. Studies tourism flows. Emphasises sustainability. Prepares for tourism industry roles.</t>
         </is>
       </c>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="6" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Master in Plasma Physics, Spectroscopy and Self-Organization</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>DEG-000015</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Applied Physics</t>
         </is>
       </c>
-      <c r="E16" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="E16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" t="inlineStr">
         <is>
           <t>Focuses on plasma diagnostics and systems behaviour. Develops analytical skills. Studies light-matter interaction. Emphasises advanced research. Prepares for physics careers.</t>
         </is>
       </c>
-      <c r="G16" s="6" t="n"/>
-      <c r="H16" s="6" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Master in Play Therapy</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>DEG-000016</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Psychotherapy</t>
         </is>
       </c>
-      <c r="E17" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="E17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" t="inlineStr">
         <is>
           <t>Focuses on therapeutic use of play for children. Develops counselling skills. Studies child psychology. Emphasises emotional development. Prepares for clinical therapy roles.</t>
         </is>
       </c>
-      <c r="G17" s="6" t="n"/>
-      <c r="H17" s="6" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Master in Podiatric Surgery</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>DEG-000017</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Surgical Medicine</t>
         </is>
       </c>
-      <c r="E18" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" t="inlineStr">
         <is>
           <t>Focuses on surgical treatment of foot disorders. Develops clinical and surgical skills. Studies anatomy and pathology. Emphasises operative care. Prepares for surgical roles.</t>
         </is>
       </c>
-      <c r="G18" s="6" t="n"/>
-      <c r="H18" s="6" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Master in Portuguese and Business</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>DEG-000018</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Business Communication</t>
         </is>
       </c>
-      <c r="E19" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="E19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" t="inlineStr">
         <is>
           <t>Focuses on Portuguese language in business contexts. Develops communication skills. Studies commerce and culture. Emphasises international trade. Prepares for business roles.</t>
         </is>
       </c>
-      <c r="G19" s="6" t="n"/>
-      <c r="H19" s="6" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Master in Post-production with Sound Design</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>DEG-000019</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Media Production</t>
         </is>
       </c>
-      <c r="E20" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="E20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" t="inlineStr">
         <is>
           <t>Focuses on audio post-production for media. Develops technical and creative skills. Studies sound design. Emphasises film and media industries. Prepares for production roles.</t>
         </is>
       </c>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="6" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Master in Power, Electronic and Telecommunication Engineering</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>DEG-000020</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Electrical Engineering</t>
         </is>
       </c>
-      <c r="E21" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="E21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" t="inlineStr">
         <is>
           <t>Focuses on integrated power and communication systems. Develops technical skills. Studies networks and electronics. Emphasises infrastructure. Prepares for engineering roles.</t>
         </is>
       </c>
-      <c r="G21" s="6" t="n"/>
-      <c r="H21" s="6" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Master in Process Engineering</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>DEG-000021</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Chemical/Industrial Engineering</t>
         </is>
       </c>
-      <c r="E22" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="inlineStr">
         <is>
           <t>Focuses on industrial process design and optimisation. Develops engineering skills. Studies production systems. Emphasises efficiency and safety. Prepares for industry roles.</t>
         </is>
       </c>
-      <c r="G22" s="6" t="n"/>
-      <c r="H22" s="6" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Master in Professional Archaeology and Comprehensive Heritage Management</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>DEG-000022</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Archaeology</t>
         </is>
       </c>
-      <c r="E23" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="E23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" t="inlineStr">
         <is>
           <t>Focuses on archaeological practice and heritage management. Develops field skills. Studies cultural preservation. Emphasises applied archaeology. Prepares for heritage roles.</t>
         </is>
       </c>
-      <c r="G23" s="6" t="n"/>
-      <c r="H23" s="6" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Master in Professional Non-surgical Aesthetic Practice</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>DEG-000023</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Aesthetic Medicine</t>
         </is>
       </c>
-      <c r="E24" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="E24" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" t="inlineStr">
         <is>
           <t>Focuses on cosmetic non-surgical treatments. Develops clinical and procedural skills. Studies skin aesthetics. Emphasises patient care. Prepares for aesthetic practice roles.</t>
         </is>
       </c>
-      <c r="G24" s="6" t="n"/>
-      <c r="H24" s="6" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Master in Professional Studies in Education</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>DEG-000024</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E25" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="inlineStr">
         <is>
           <t>Focuses on advanced teaching and learning practice. Develops pedagogical skills. Studies education systems. Emphasises instructional improvement. Prepares for educator roles.</t>
         </is>
       </c>
-      <c r="G25" s="6" t="n"/>
-      <c r="H25" s="6" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Master in Professional Translation Studies</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>DEG-000025</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Translation Studies</t>
         </is>
       </c>
-      <c r="E26" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="E26" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" t="inlineStr">
         <is>
           <t>Focuses on advanced translation theory and practice. Develops language skills. Studies translation techniques. Emphasises accuracy and fluency. Prepares for translator roles.</t>
         </is>
       </c>
-      <c r="G26" s="6" t="n"/>
-      <c r="H26" s="6" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Master in Prostate Cancer Care</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>DEG-000026</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Oncology</t>
         </is>
       </c>
-      <c r="E27" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="inlineStr">
         <is>
           <t>Focuses on diagnosis and treatment of prostate cancer. Develops clinical skills. Studies oncology care pathways. Emphasises patient management. Prepares for healthcare roles.</t>
         </is>
       </c>
-      <c r="G27" s="6" t="n"/>
-      <c r="H27" s="6" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Master in Psychology Conversion</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>DEG-000027</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Conversion Psychology</t>
         </is>
       </c>
-      <c r="E28" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="E28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="inlineStr">
         <is>
           <t>Focuses on foundational psychology training. Develops core analytical skills. Studies psychological theory. Emphasises transition into field. Prepares for psychology careers.</t>
         </is>
       </c>
-      <c r="G28" s="6" t="n"/>
-      <c r="H28" s="6" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>Master in Psycho-oncology and Palliative Care</t>
         </is>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>DEG-000028</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Health Psychology</t>
         </is>
       </c>
-      <c r="E29" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="inlineStr">
         <is>
           <t>Focuses on psychological support in cancer care. Develops clinical intervention skills. Studies patient wellbeing. Emphasises end-of-life care. Prepares for healthcare roles.</t>
         </is>
       </c>
-      <c r="G29" s="6" t="n"/>
-      <c r="H29" s="6" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>Master in Public Health, Public Health Nutrition and Epidemiology</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>DEG-000029</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>Public Health Nutrition</t>
         </is>
       </c>
-      <c r="E30" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="inlineStr">
         <is>
           <t>Focuses on nutrition and disease prevention. Develops epidemiological skills. Studies diet and population health. Emphasises prevention strategies. Prepares for health roles.</t>
         </is>
       </c>
-      <c r="G30" s="6" t="n"/>
-      <c r="H30" s="6" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>Bachelor of Design in Visual Communication and BA in International Studies</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>DEG-000030</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Design / Communication</t>
         </is>
       </c>
-      <c r="E31" s="6" t="n">
+      <c r="E31" t="n">
         <v>4</v>
       </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>Combines visual communication with global studies. Covers branding and media. Develops creative skills. Prepares for design careers.</t>
         </is>
       </c>
-      <c r="G31" s="6" t="n"/>
-      <c r="H31" s="6" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Bachelor of Teaching and BA in Mathematics</t>
         </is>
       </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>DEG-000031</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Education / Mathematics</t>
         </is>
       </c>
-      <c r="E32" s="6" t="n">
+      <c r="E32" t="n">
         <v>4</v>
       </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>Combines teaching with mathematics. Covers pedagogy and quantitative skills. Develops instructional ability. Prepares for teaching roles.</t>
         </is>
       </c>
-      <c r="G32" s="6" t="n"/>
-      <c r="H32" s="6" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Bachelor of Health Science in Traditional Chinese Medicine and BA in International Studies</t>
         </is>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>DEG-000032</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Health / Traditional Medicine</t>
         </is>
       </c>
-      <c r="E33" s="6" t="n">
+      <c r="E33" t="n">
         <v>4</v>
       </c>
-      <c r="F33" s="6" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>Combines Chinese medicine with global studies. Covers holistic health systems. Develops clinical knowledge. Prepares for healthcare roles.</t>
         </is>
       </c>
-      <c r="G33" s="6" t="n"/>
-      <c r="H33" s="6" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>Bachelor of Teaching and BA in Visual Arts</t>
         </is>
       </c>
-      <c r="B34" s="6" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>DEG-000033</t>
         </is>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Education / Arts</t>
         </is>
       </c>
-      <c r="E34" s="6" t="n">
+      <c r="E34" t="n">
         <v>4</v>
       </c>
-      <c r="F34" s="6" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Combines teaching with visual arts practice. Covers pedagogy and creativity. Develops instructional skills. Prepares for arts education roles.</t>
         </is>
       </c>
-      <c r="G34" s="6" t="n"/>
-      <c r="H34" s="6" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>Bachelor of Education and BA in International Studies</t>
         </is>
       </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>DEG-000034</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E35" s="6" t="n">
+      <c r="E35" t="n">
         <v>4</v>
       </c>
-      <c r="F35" s="6" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>Combines teaching qualifications with global studies. Covers pedagogy and culture. Develops instructional skills. Prepares for education roles.</t>
         </is>
       </c>
-      <c r="G35" s="6" t="n"/>
-      <c r="H35" s="6" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>Bachelor of Teaching and BA in Technology</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>DEG-000035</t>
         </is>
       </c>
-      <c r="C36" s="6" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>Education / Technology</t>
         </is>
       </c>
-      <c r="E36" s="6" t="n">
+      <c r="E36" t="n">
         <v>4</v>
       </c>
-      <c r="F36" s="6" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>Combines teaching with technology studies. Covers digital tools and pedagogy. Develops instructional skills. Prepares for STEM education roles.</t>
         </is>
       </c>
-      <c r="G36" s="6" t="n"/>
-      <c r="H36" s="6" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>Bachelor of Journalism and Professional Writing and BA in Creative Writing and Literature</t>
         </is>
       </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>DEG-000036</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>Journalism / Writing</t>
         </is>
       </c>
-      <c r="E37" s="6" t="n">
+      <c r="E37" t="n">
         <v>4</v>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>Combines journalism with creative writing. Covers reporting, storytelling, and media. Develops communication skills. Prepares for media careers.</t>
         </is>
       </c>
-      <c r="G37" s="6" t="n"/>
-      <c r="H37" s="6" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>Bachelor of Commerce, BA in Psychology</t>
         </is>
       </c>
-      <c r="B38" s="6" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>DEG-000037</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>Business / Psychology</t>
         </is>
       </c>
-      <c r="E38" s="6" t="n">
+      <c r="E38" t="n">
         <v>4</v>
       </c>
-      <c r="F38" s="6" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>Combines commerce with psychology studies. Covers business strategy and human behaviour. Develops analytical skills. Prepares for corporate roles.</t>
         </is>
       </c>
-      <c r="G38" s="6" t="n"/>
-      <c r="H38" s="6" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>Bachelor of Nursing and BA in International Studies</t>
         </is>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>DEG-000038</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>Nursing</t>
         </is>
       </c>
-      <c r="E39" s="6" t="n">
+      <c r="E39" t="n">
         <v>4</v>
       </c>
-      <c r="F39" s="6" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>Combines nursing practice with global studies. Covers healthcare systems and patient care. Develops clinical skills. Prepares for nursing careers.</t>
         </is>
       </c>
-      <c r="G39" s="6" t="n"/>
-      <c r="H39" s="6" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
+      <c r="A40" t="inlineStr">
         <is>
           <t>Bachelor of Teaching and BA in Humanities</t>
         </is>
       </c>
-      <c r="B40" s="6" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>DEG-000039</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E40" s="6" t="n">
+      <c r="E40" t="n">
         <v>4</v>
       </c>
-      <c r="F40" s="6" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>Combines teaching qualification with humanities studies. Covers pedagogy and culture. Develops instructional skills. Prepares for education roles.</t>
         </is>
       </c>
-      <c r="G40" s="6" t="n"/>
-      <c r="H40" s="6" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="inlineStr">
+      <c r="A41" t="inlineStr">
         <is>
           <t>Bachelor of Design in Interior Architecture and BA in International Studies</t>
         </is>
       </c>
-      <c r="B41" s="6" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>DEG-000040</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>Design / Architecture</t>
         </is>
       </c>
-      <c r="E41" s="6" t="n">
+      <c r="E41" t="n">
         <v>4</v>
       </c>
-      <c r="F41" s="6" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>Combines interior design with global studies. Covers spatial design and culture. Develops creative and technical skills. Prepares for design careers.</t>
         </is>
       </c>
-      <c r="G41" s="6" t="n"/>
-      <c r="H41" s="6" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="inlineStr">
+      <c r="A42" t="inlineStr">
         <is>
           <t>Bachelor of Design in Product Design and BA in International Studies</t>
         </is>
       </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>DEG-000041</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>Design / Product</t>
         </is>
       </c>
-      <c r="E42" s="6" t="n">
+      <c r="E42" t="n">
         <v>4</v>
       </c>
-      <c r="F42" s="6" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>Combines product design with global studies. Covers innovation and user-centred design. Develops technical skills. Prepares for design industry roles.</t>
         </is>
       </c>
-      <c r="G42" s="6" t="n"/>
-      <c r="H42" s="6" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="inlineStr">
+      <c r="A43" t="inlineStr">
         <is>
           <t>Bachelor of Medical Science and BA in International Studies</t>
         </is>
       </c>
-      <c r="B43" s="6" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>DEG-000042</t>
         </is>
       </c>
-      <c r="C43" s="6" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>Medical Science</t>
         </is>
       </c>
-      <c r="E43" s="6" t="n">
+      <c r="E43" t="n">
         <v>4</v>
       </c>
-      <c r="F43" s="6" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>Combines medical science with global studies. Covers biology, health systems, and policy. Develops scientific skills. Prepares for health sector roles.</t>
         </is>
       </c>
-      <c r="G43" s="6" t="n"/>
-      <c r="H43" s="6" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="inlineStr">
+      <c r="A44" t="inlineStr">
         <is>
           <t>Bachelor of Design in Animation and BA in International Studies</t>
         </is>
       </c>
-      <c r="B44" s="6" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>DEG-000043</t>
         </is>
       </c>
-      <c r="C44" s="6" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D44" s="6" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>Design / International Studies</t>
         </is>
       </c>
-      <c r="E44" s="6" t="n">
+      <c r="E44" t="n">
         <v>4</v>
       </c>
-      <c r="F44" s="6" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>Combines animation with global cultural studies. Covers storytelling and media production. Develops creative skills. Prepares for animation and media roles.</t>
         </is>
       </c>
-      <c r="G44" s="6" t="n"/>
-      <c r="H44" s="6" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="inlineStr">
+      <c r="A45" t="inlineStr">
         <is>
           <t>Bachelor of Design in Photography and BA in International Studies</t>
         </is>
       </c>
-      <c r="B45" s="6" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>DEG-000044</t>
         </is>
       </c>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D45" s="6" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Design / Photography</t>
         </is>
       </c>
-      <c r="E45" s="6" t="n">
+      <c r="E45" t="n">
         <v>4</v>
       </c>
-      <c r="F45" s="6" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>Combines photography with international studies. Covers visual storytelling and culture. Develops artistic skills. Prepares for media and photography roles.</t>
         </is>
       </c>
-      <c r="G45" s="6" t="n"/>
-      <c r="H45" s="6" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="inlineStr">
+      <c r="A46" t="inlineStr">
         <is>
           <t>Bachelor of Commerce and BA in Psychology and Economics</t>
         </is>
       </c>
-      <c r="B46" s="6" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>DEG-000045</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>Business / Social Science</t>
         </is>
       </c>
-      <c r="E46" s="6" t="n">
+      <c r="E46" t="n">
         <v>4</v>
       </c>
-      <c r="F46" s="6" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>Integrates commerce, psychology, and economics. Covers markets, behaviour, and policy. Develops analytical skills. Prepares for finance and consulting roles.</t>
         </is>
       </c>
-      <c r="G46" s="6" t="n"/>
-      <c r="H46" s="6" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="inlineStr">
+      <c r="A47" t="inlineStr">
         <is>
           <t>Bachelor of Communication in Creative Writing and BA in International Studies</t>
         </is>
       </c>
-      <c r="B47" s="6" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>DEG-000046</t>
         </is>
       </c>
-      <c r="C47" s="6" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D47" s="6" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>Communication / International Studies</t>
         </is>
       </c>
-      <c r="E47" s="6" t="n">
+      <c r="E47" t="n">
         <v>4</v>
       </c>
-      <c r="F47" s="6" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>Combines creative writing with global studies. Covers media, culture, and communication. Develops storytelling skills. Prepares for media and international roles.</t>
         </is>
       </c>
-      <c r="G47" s="6" t="n"/>
-      <c r="H47" s="6" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="inlineStr">
+      <c r="A48" t="inlineStr">
         <is>
           <t>Bachelor of Construction Project Management, BA in International Studies</t>
         </is>
       </c>
-      <c r="B48" s="6" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>DEG-000047</t>
         </is>
       </c>
-      <c r="C48" s="6" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D48" s="6" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>Construction / International Studies</t>
         </is>
       </c>
-      <c r="E48" s="6" t="n">
+      <c r="E48" t="n">
         <v>4</v>
       </c>
-      <c r="F48" s="6" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>Combines construction management with global studies. Covers planning, infrastructure, and policy. Develops leadership skills. Prepares for project management roles.</t>
         </is>
       </c>
-      <c r="G48" s="6" t="n"/>
-      <c r="H48" s="6" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="inlineStr">
+      <c r="A49" t="inlineStr">
         <is>
           <t>Bachelor of Commerce and BA in Psychology</t>
         </is>
       </c>
-      <c r="B49" s="6" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>DEG-000048</t>
         </is>
       </c>
-      <c r="C49" s="6" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>Business / Psychology</t>
         </is>
       </c>
-      <c r="E49" s="6" t="n">
+      <c r="E49" t="n">
         <v>4</v>
       </c>
-      <c r="F49" s="6" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>Combines business commerce with psychological science. Covers markets, behaviour, and analytics. Develops interdisciplinary skills. Prepares for business and HR roles.</t>
         </is>
       </c>
-      <c r="G49" s="6" t="n"/>
-      <c r="H49" s="6" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="inlineStr">
+      <c r="A50" t="inlineStr">
         <is>
           <t>Bachelor in Transfer Degree</t>
         </is>
       </c>
-      <c r="B50" s="6" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>DEG-000049</t>
         </is>
       </c>
-      <c r="C50" s="6" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D50" s="6" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>General Studies</t>
         </is>
       </c>
-      <c r="E50" s="6" t="n">
+      <c r="E50" t="n">
         <v>4</v>
       </c>
-      <c r="F50" s="6" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>Provides foundational academic coursework for transfer. Develops core academic skills. Focuses on university progression pathways. Prepares students for advanced degrees.</t>
         </is>
       </c>
-      <c r="G50" s="6" t="n"/>
-      <c r="H50" s="6" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="inlineStr">
+      <c r="A51" t="inlineStr">
         <is>
           <t>Bachelor and MBA in Supply Chain Management</t>
         </is>
       </c>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>DEG-000050</t>
         </is>
       </c>
-      <c r="C51" s="6" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D51" s="6" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>Business / Logistics</t>
         </is>
       </c>
-      <c r="E51" s="6" t="n">
+      <c r="E51" t="n">
         <v>4</v>
       </c>
-      <c r="F51" s="6" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>Integrated program covering supply chain and advanced business management. Covers logistics, operations, and strategy. Develops leadership skills. Prepares for senior management roles.</t>
         </is>
       </c>
-      <c r="G51" s="6" t="n"/>
-      <c r="H51" s="6" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="inlineStr">
+      <c r="A52" t="inlineStr">
         <is>
           <t>Bachelor of Law with English Language Studies</t>
         </is>
       </c>
-      <c r="B52" s="6" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>DEG-000051</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D52" s="6" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>English Studies</t>
         </is>
       </c>
-      <c r="E52" s="6" t="n">
+      <c r="E52" t="n">
         <v>4</v>
       </c>
-      <c r="F52" s="6" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>Combines law with advanced study of English linguistics and usage. Builds strong written and verbal reasoning. Prepares for careers in law, media, publishing, or public administration.</t>
         </is>
       </c>
-      <c r="G52" s="6" t="n"/>
-      <c r="H52" s="6" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="inlineStr">
+      <c r="A53" t="inlineStr">
         <is>
           <t>Bachelor of Law with English</t>
         </is>
       </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>DEG-000052</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D53" s="6" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="E53" s="6" t="n">
+      <c r="E53" t="n">
         <v>4</v>
       </c>
-      <c r="F53" s="6" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>Combines law with English language and literature studies. Strengthens critical thinking, analysis, and communication. Prepares for careers in law, publishing, education, or media industries.</t>
         </is>
       </c>
-      <c r="G53" s="6" t="n"/>
-      <c r="H53" s="6" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="inlineStr">
+      <c r="A54" t="inlineStr">
         <is>
           <t>Bachelor of Law with Classical Studies</t>
         </is>
       </c>
-      <c r="B54" s="6" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>DEG-000053</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D54" s="6" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>Classical Studies</t>
         </is>
       </c>
-      <c r="E54" s="6" t="n">
+      <c r="E54" t="n">
         <v>4</v>
       </c>
-      <c r="F54" s="6" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>Integrates law with ancient Greek and Roman civilizations. Develops analytical and historical interpretation skills. Prepares for careers in law, academia, heritage, or cultural policy sectors.</t>
         </is>
       </c>
-      <c r="G54" s="6" t="n"/>
-      <c r="H54" s="6" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="inlineStr">
+      <c r="A55" t="inlineStr">
         <is>
           <t>Bachelor of Law with Criminology</t>
         </is>
       </c>
-      <c r="B55" s="6" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>DEG-000054</t>
         </is>
       </c>
-      <c r="C55" s="6" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D55" s="6" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>Criminology</t>
         </is>
       </c>
-      <c r="E55" s="6" t="n">
+      <c r="E55" t="n">
         <v>4</v>
       </c>
-      <c r="F55" s="6" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>Combines law with the study of crime, justice, and society. Develops understanding of criminal behavior and legal responses. Leads to careers in policing, legal practice, or criminal justice policy.</t>
         </is>
       </c>
-      <c r="G55" s="6" t="n"/>
-      <c r="H55" s="6" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="inlineStr">
+      <c r="A56" t="inlineStr">
         <is>
           <t>Bachelor of Forestry Transfer</t>
         </is>
       </c>
-      <c r="B56" s="6" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>DEG-000055</t>
         </is>
       </c>
-      <c r="C56" s="6" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D56" s="6" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>Forestry (Transfer Program)</t>
         </is>
       </c>
-      <c r="E56" s="6" t="n">
+      <c r="E56" t="n">
         <v>4</v>
       </c>
-      <c r="F56" s="6" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>Provides foundational forestry education for academic transfer pathways. Develops basic ecological and scientific skills. Prepares students for advanced forestry studies. Strengthens academic readiness. Supports progression into specialized forestry degrees.</t>
         </is>
       </c>
-      <c r="G56" s="6" t="n"/>
-      <c r="H56" s="6" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="inlineStr">
+      <c r="A57" t="inlineStr">
         <is>
           <t>Bachelor of Language and Literature Education</t>
         </is>
       </c>
-      <c r="B57" s="6" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>DEG-000056</t>
         </is>
       </c>
-      <c r="C57" s="6" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D57" s="6" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>Education &amp; Language</t>
         </is>
       </c>
-      <c r="E57" s="6" t="n">
+      <c r="E57" t="n">
         <v>4</v>
       </c>
-      <c r="F57" s="6" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>Focuses on teaching languages and literature. Builds pedagogy and communication skills. Graduates work as language teachers.</t>
         </is>
       </c>
-      <c r="G57" s="6" t="n"/>
-      <c r="H57" s="6" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="inlineStr">
+      <c r="A58" t="inlineStr">
         <is>
           <t>Bachelor of Mathematics with Education</t>
         </is>
       </c>
-      <c r="B58" s="6" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>DEG-000057</t>
         </is>
       </c>
-      <c r="C58" s="6" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D58" s="6" t="inlineStr">
+      <c r="D58" t="inlineStr">
         <is>
           <t>Mathematics Education</t>
         </is>
       </c>
-      <c r="E58" s="6" t="n">
+      <c r="E58" t="n">
         <v>4</v>
       </c>
-      <c r="F58" s="6" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>Focuses on mathematics teaching and learning methods. Builds pedagogical skills. Graduates work in schools or education roles.</t>
         </is>
       </c>
-      <c r="G58" s="6" t="n"/>
-      <c r="H58" s="6" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="inlineStr">
+      <c r="A59" t="inlineStr">
         <is>
           <t>Bachelor of Italian and Persian</t>
         </is>
       </c>
-      <c r="B59" s="6" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>DEG-000058</t>
         </is>
       </c>
-      <c r="C59" s="6" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D59" s="6" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>Language Studies</t>
         </is>
       </c>
-      <c r="E59" s="6" t="n">
+      <c r="E59" t="n">
         <v>4</v>
       </c>
-      <c r="F59" s="6" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>Combines Italian and Persian languages. Builds intercultural communication skills. Graduates work in translation and diplomacy.</t>
         </is>
       </c>
-      <c r="G59" s="6" t="n"/>
-      <c r="H59" s="6" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="inlineStr">
+      <c r="A60" t="inlineStr">
         <is>
           <t>Bachelor of Medical Studies and Doctor of Medicine</t>
         </is>
       </c>
-      <c r="B60" s="6" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>DEG-000059</t>
         </is>
       </c>
-      <c r="C60" s="6" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D60" s="6" t="inlineStr">
+      <c r="D60" t="inlineStr">
         <is>
           <t>Medical Pathway</t>
         </is>
       </c>
-      <c r="E60" s="6" t="n">
+      <c r="E60" t="n">
         <v>4</v>
       </c>
-      <c r="F60" s="6" t="inlineStr">
+      <c r="F60" t="inlineStr">
         <is>
           <t>Integrated medical training program. Builds clinical and scientific expertise. Graduates become licensed medical practitioners.</t>
         </is>
       </c>
-      <c r="G60" s="6" t="n"/>
-      <c r="H60" s="6" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="6" t="inlineStr">
+      <c r="A61" t="inlineStr">
         <is>
           <t>Bachelor of History Teaching</t>
         </is>
       </c>
-      <c r="B61" s="6" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>DEG-000060</t>
         </is>
       </c>
-      <c r="C61" s="6" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D61" s="6" t="inlineStr">
+      <c r="D61" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E61" s="6" t="n">
+      <c r="E61" t="n">
         <v>4</v>
       </c>
-      <c r="F61" s="6" t="inlineStr">
+      <c r="F61" t="inlineStr">
         <is>
           <t>Studies methods of teaching history. Develops pedagogical skills. Focuses on classroom instruction. Graduates work as educators.</t>
         </is>
       </c>
-      <c r="G61" s="6" t="n"/>
-      <c r="H61" s="6" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="6" t="inlineStr">
+      <c r="A62" t="inlineStr">
         <is>
           <t>PhD in Fluids Engineering</t>
         </is>
       </c>
-      <c r="B62" s="6" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>DEG-000061</t>
         </is>
       </c>
-      <c r="C62" s="6" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D62" s="6" t="inlineStr">
+      <c r="D62" t="inlineStr">
         <is>
           <t>Mechanical Engineering</t>
         </is>
       </c>
-      <c r="E62" s="6" t="n">
+      <c r="E62" t="n">
         <v>3</v>
       </c>
-      <c r="F62" s="6" t="inlineStr">
+      <c r="F62" t="inlineStr">
         <is>
           <t>Studies fluid flow and engineering system design. Develops expertise in computational modeling and experimental research. Focuses on industrial and energy applications. Graduates work in research, aerospace, and engineering firms.</t>
         </is>
       </c>
-      <c r="G62" s="6" t="n"/>
-      <c r="H62" s="6" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="6" t="inlineStr">
+      <c r="A63" t="inlineStr">
         <is>
           <t>PhD in Food and Biochemical Technology</t>
         </is>
       </c>
-      <c r="B63" s="6" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>DEG-000062</t>
         </is>
       </c>
-      <c r="C63" s="6" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D63" s="6" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>Food Science</t>
         </is>
       </c>
-      <c r="E63" s="6" t="n">
+      <c r="E63" t="n">
         <v>3</v>
       </c>
-      <c r="F63" s="6" t="inlineStr">
+      <c r="F63" t="inlineStr">
         <is>
           <t>Combines food science with biochemical technologies. Develops expertise in food processing and biochemical research. Focuses on improving food quality and innovation. Graduates work in academia, biotechnology, and food industries.</t>
         </is>
       </c>
-      <c r="G63" s="6" t="n"/>
-      <c r="H63" s="6" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="6" t="inlineStr">
+      <c r="A64" t="inlineStr">
         <is>
           <t>PhD in Food Systems</t>
         </is>
       </c>
-      <c r="B64" s="6" t="inlineStr">
+      <c r="B64" t="inlineStr">
         <is>
           <t>DEG-000063</t>
         </is>
       </c>
-      <c r="C64" s="6" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D64" s="6" t="inlineStr">
+      <c r="D64" t="inlineStr">
         <is>
           <t>Food Systems</t>
         </is>
       </c>
-      <c r="E64" s="6" t="n">
+      <c r="E64" t="n">
         <v>3</v>
       </c>
-      <c r="F64" s="6" t="inlineStr">
+      <c r="F64" t="inlineStr">
         <is>
           <t>Explores food production, distribution, and consumption systems. Develops interdisciplinary research and policy skills. Focuses on sustainability and resilience. Graduates work in academia, government, and nonprofit organizations.</t>
         </is>
       </c>
-      <c r="G64" s="6" t="n"/>
-      <c r="H64" s="6" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="inlineStr">
+      <c r="A65" t="inlineStr">
         <is>
           <t>PhD in Gender Studies</t>
         </is>
       </c>
-      <c r="B65" s="6" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>DEG-000064</t>
         </is>
       </c>
-      <c r="C65" s="6" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D65" s="6" t="inlineStr">
+      <c r="D65" t="inlineStr">
         <is>
           <t>Gender Studies</t>
         </is>
       </c>
-      <c r="E65" s="6" t="n">
+      <c r="E65" t="n">
         <v>3</v>
       </c>
-      <c r="F65" s="6" t="inlineStr">
+      <c r="F65" t="inlineStr">
         <is>
           <t>Explores gender through social, political, and cultural research. Develops critical thinking and interdisciplinary research skills. Focuses on identity and equality. Graduates work in academia, policy, and community organizations.</t>
         </is>
       </c>
-      <c r="G65" s="6" t="n"/>
-      <c r="H65" s="6" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="6" t="inlineStr">
+      <c r="A66" t="inlineStr">
         <is>
           <t>PhD in Geodesy and Geoinformatics</t>
         </is>
       </c>
-      <c r="B66" s="6" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t>DEG-000065</t>
         </is>
       </c>
-      <c r="C66" s="6" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D66" s="6" t="inlineStr">
+      <c r="D66" t="inlineStr">
         <is>
           <t>Geospatial Science</t>
         </is>
       </c>
-      <c r="E66" s="6" t="n">
+      <c r="E66" t="n">
         <v>3</v>
       </c>
-      <c r="F66" s="6" t="inlineStr">
+      <c r="F66" t="inlineStr">
         <is>
           <t>Combines geodesy with digital geographic information systems. Develops expertise in spatial analysis and geospatial technologies. Focuses on Earth measurement and mapping. Graduates work in academia, surveying, and GIS industries.</t>
         </is>
       </c>
-      <c r="G66" s="6" t="n"/>
-      <c r="H66" s="6" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="6" t="inlineStr">
+      <c r="A67" t="inlineStr">
         <is>
           <t>PhD in Geography and Earth Science</t>
         </is>
       </c>
-      <c r="B67" s="6" t="inlineStr">
+      <c r="B67" t="inlineStr">
         <is>
           <t>DEG-000066</t>
         </is>
       </c>
-      <c r="C67" s="6" t="inlineStr">
+      <c r="C67" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D67" s="6" t="inlineStr">
+      <c r="D67" t="inlineStr">
         <is>
           <t>Earth Science</t>
         </is>
       </c>
-      <c r="E67" s="6" t="n">
+      <c r="E67" t="n">
         <v>3</v>
       </c>
-      <c r="F67" s="6" t="inlineStr">
+      <c r="F67" t="inlineStr">
         <is>
           <t>Combines geography with Earth science research. Develops expertise in environmental systems and geospatial analysis. Focuses on understanding Earth's processes. Graduates work in academia, environmental consulting, and government.</t>
         </is>
       </c>
-      <c r="G67" s="6" t="n"/>
-      <c r="H67" s="6" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="6" t="inlineStr">
+      <c r="A68" t="inlineStr">
         <is>
           <t>PhD in Geometry and Topology</t>
         </is>
       </c>
-      <c r="B68" s="6" t="inlineStr">
+      <c r="B68" t="inlineStr">
         <is>
           <t>DEG-000067</t>
         </is>
       </c>
-      <c r="C68" s="6" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D68" s="6" t="inlineStr">
+      <c r="D68" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="E68" s="6" t="n">
+      <c r="E68" t="n">
         <v>3</v>
       </c>
-      <c r="F68" s="6" t="inlineStr">
+      <c r="F68" t="inlineStr">
         <is>
           <t>Studies the properties and structures of geometric spaces. Develops expertise in abstract mathematics and theoretical research. Focuses on advanced mathematical concepts. Graduates work in academia, research, and higher education.</t>
         </is>
       </c>
-      <c r="G68" s="6" t="n"/>
-      <c r="H68" s="6" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="6" t="inlineStr">
+      <c r="A69" t="inlineStr">
         <is>
           <t>PhD in Geospatial Analytics</t>
         </is>
       </c>
-      <c r="B69" s="6" t="inlineStr">
+      <c r="B69" t="inlineStr">
         <is>
           <t>DEG-000068</t>
         </is>
       </c>
-      <c r="C69" s="6" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D69" s="6" t="inlineStr">
+      <c r="D69" t="inlineStr">
         <is>
           <t>Data Science</t>
         </is>
       </c>
-      <c r="E69" s="6" t="n">
+      <c r="E69" t="n">
         <v>3</v>
       </c>
-      <c r="F69" s="6" t="inlineStr">
+      <c r="F69" t="inlineStr">
         <is>
           <t>Studies advanced analysis of geographic and spatial data. Develops expertise in GIS, machine learning, and predictive modeling. Focuses on spatial decision-making. Graduates work in academia, government, and technology industries.</t>
         </is>
       </c>
-      <c r="G69" s="6" t="n"/>
-      <c r="H69" s="6" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="6" t="inlineStr">
+      <c r="A70" t="inlineStr">
         <is>
           <t>PhD in Grain Science</t>
         </is>
       </c>
-      <c r="B70" s="6" t="inlineStr">
+      <c r="B70" t="inlineStr">
         <is>
           <t>DEG-000069</t>
         </is>
       </c>
-      <c r="C70" s="6" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D70" s="6" t="inlineStr">
+      <c r="D70" t="inlineStr">
         <is>
           <t>Agricultural Science</t>
         </is>
       </c>
-      <c r="E70" s="6" t="n">
+      <c r="E70" t="n">
         <v>3</v>
       </c>
-      <c r="F70" s="6" t="inlineStr">
+      <c r="F70" t="inlineStr">
         <is>
           <t>Studies grain production, processing, and quality. Develops expertise in cereal chemistry and agricultural research. Focuses on food quality and sustainable production. Graduates work in academia, agriculture, and food industries.</t>
         </is>
       </c>
-      <c r="G70" s="6" t="n"/>
-      <c r="H70" s="6" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="6" t="inlineStr">
+      <c r="A71" t="inlineStr">
         <is>
           <t>PhD in Health Economics and Policy</t>
         </is>
       </c>
-      <c r="B71" s="6" t="inlineStr">
+      <c r="B71" t="inlineStr">
         <is>
           <t>DEG-000070</t>
         </is>
       </c>
-      <c r="C71" s="6" t="inlineStr">
+      <c r="C71" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D71" s="6" t="inlineStr">
+      <c r="D71" t="inlineStr">
         <is>
           <t>Health Economics</t>
         </is>
       </c>
-      <c r="E71" s="6" t="n">
+      <c r="E71" t="n">
         <v>3</v>
       </c>
-      <c r="F71" s="6" t="inlineStr">
+      <c r="F71" t="inlineStr">
         <is>
           <t>Integrates economic analysis with healthcare policy research. Develops expertise in health financing and policy evaluation. Focuses on improving health systems. Graduates work in academia, government, and healthcare organizations.</t>
         </is>
       </c>
-      <c r="G71" s="6" t="n"/>
-      <c r="H71" s="6" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="6" t="inlineStr">
+      <c r="A72" t="inlineStr">
         <is>
           <t>PhD in Hispanic Studies and Comparative Literature</t>
         </is>
       </c>
-      <c r="B72" s="6" t="inlineStr">
+      <c r="B72" t="inlineStr">
         <is>
           <t>DEG-000071</t>
         </is>
       </c>
-      <c r="C72" s="6" t="inlineStr">
+      <c r="C72" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D72" s="6" t="inlineStr">
+      <c r="D72" t="inlineStr">
         <is>
           <t>Literature</t>
         </is>
       </c>
-      <c r="E72" s="6" t="n">
+      <c r="E72" t="n">
         <v>3</v>
       </c>
-      <c r="F72" s="6" t="inlineStr">
+      <c r="F72" t="inlineStr">
         <is>
           <t>Combines Hispanic studies with comparative literary research. Develops expertise in literary analysis and cross-cultural interpretation. Focuses on global literary traditions. Graduates work in academia, publishing, and education.</t>
         </is>
       </c>
-      <c r="G72" s="6" t="n"/>
-      <c r="H72" s="6" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="6" t="inlineStr">
+      <c r="A73" t="inlineStr">
         <is>
           <t>PhD in History of Art and Archaeology</t>
         </is>
       </c>
-      <c r="B73" s="6" t="inlineStr">
+      <c r="B73" t="inlineStr">
         <is>
           <t>DEG-000072</t>
         </is>
       </c>
-      <c r="C73" s="6" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D73" s="6" t="inlineStr">
+      <c r="D73" t="inlineStr">
         <is>
           <t>Art History</t>
         </is>
       </c>
-      <c r="E73" s="6" t="n">
+      <c r="E73" t="n">
         <v>3</v>
       </c>
-      <c r="F73" s="6" t="inlineStr">
+      <c r="F73" t="inlineStr">
         <is>
           <t>Combines art history with archaeological research. Develops expertise in material culture and historical interpretation. Focuses on ancient and historical artifacts. Graduates work in academia, museums, and heritage organizations.</t>
         </is>
       </c>
-      <c r="G73" s="6" t="n"/>
-      <c r="H73" s="6" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="6" t="inlineStr">
+      <c r="A74" t="inlineStr">
         <is>
           <t>PhD in Laser, Photonics and Vision</t>
         </is>
       </c>
-      <c r="B74" s="6" t="inlineStr">
+      <c r="B74" t="inlineStr">
         <is>
           <t>DEG-000073</t>
         </is>
       </c>
-      <c r="C74" s="6" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D74" s="6" t="inlineStr">
+      <c r="D74" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="E74" s="6" t="n">
+      <c r="E74" t="n">
         <v>3</v>
       </c>
-      <c r="F74" s="6" t="inlineStr">
+      <c r="F74" t="inlineStr">
         <is>
           <t>Studies laser systems, photonics, and optical vision technologies. Develops expertise in optics, imaging, and applied physics. Focuses on light-based technologies. Graduates work in academia, research labs, and optical industries.</t>
         </is>
       </c>
-      <c r="G74" s="6" t="n"/>
-      <c r="H74" s="6" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="6" t="inlineStr">
+      <c r="A75" t="inlineStr">
         <is>
           <t>PhD in Latin American Cultural Studies</t>
         </is>
       </c>
-      <c r="B75" s="6" t="inlineStr">
+      <c r="B75" t="inlineStr">
         <is>
           <t>DEG-000074</t>
         </is>
       </c>
-      <c r="C75" s="6" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D75" s="6" t="inlineStr">
+      <c r="D75" t="inlineStr">
         <is>
           <t>Cultural Studies</t>
         </is>
       </c>
-      <c r="E75" s="6" t="n">
+      <c r="E75" t="n">
         <v>3</v>
       </c>
-      <c r="F75" s="6" t="inlineStr">
+      <c r="F75" t="inlineStr">
         <is>
           <t>Explores cultural production, identity, and history in Latin America. Develops expertise in literary and cultural theory. Focuses on regional cultural expression. Graduates work in academia, publishing, and cultural organizations.</t>
         </is>
       </c>
-      <c r="G75" s="6" t="n"/>
-      <c r="H75" s="6" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="6" t="inlineStr">
+      <c r="A76" t="inlineStr">
         <is>
           <t>PhD in Leadership and Policy Studies in Education</t>
         </is>
       </c>
-      <c r="B76" s="6" t="inlineStr">
+      <c r="B76" t="inlineStr">
         <is>
           <t>DEG-000075</t>
         </is>
       </c>
-      <c r="C76" s="6" t="inlineStr">
+      <c r="C76" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D76" s="6" t="inlineStr">
+      <c r="D76" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E76" s="6" t="n">
+      <c r="E76" t="n">
         <v>3</v>
       </c>
-      <c r="F76" s="6" t="inlineStr">
+      <c r="F76" t="inlineStr">
         <is>
           <t>Examines leadership and policy in educational systems. Develops expertise in administration, policy analysis, and school leadership. Focuses on educational improvement. Graduates work in academia, schools, and government agencies.</t>
         </is>
       </c>
-      <c r="G76" s="6" t="n"/>
-      <c r="H76" s="6" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="6" t="inlineStr">
+      <c r="A77" t="inlineStr">
         <is>
           <t>PhD in Management Finance</t>
         </is>
       </c>
-      <c r="B77" s="6" t="inlineStr">
+      <c r="B77" t="inlineStr">
         <is>
           <t>DEG-000076</t>
         </is>
       </c>
-      <c r="C77" s="6" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D77" s="6" t="inlineStr">
+      <c r="D77" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="E77" s="6" t="n">
+      <c r="E77" t="n">
         <v>3</v>
       </c>
-      <c r="F77" s="6" t="inlineStr">
+      <c r="F77" t="inlineStr">
         <is>
           <t>Integrates financial management with organizational strategy. Develops expertise in corporate finance, investment, and risk management. Focuses on financial decision-making. Graduates work in finance, corporations, and consulting.</t>
         </is>
       </c>
-      <c r="G77" s="6" t="n"/>
-      <c r="H77" s="6" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="6" t="inlineStr">
+      <c r="A78" t="inlineStr">
         <is>
           <t>PhD in Marine Engine Engineering</t>
         </is>
       </c>
-      <c r="B78" s="6" t="inlineStr">
+      <c r="B78" t="inlineStr">
         <is>
           <t>DEG-000077</t>
         </is>
       </c>
-      <c r="C78" s="6" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D78" s="6" t="inlineStr">
+      <c r="D78" t="inlineStr">
         <is>
           <t>Marine Engineering</t>
         </is>
       </c>
-      <c r="E78" s="6" t="n">
+      <c r="E78" t="n">
         <v>3</v>
       </c>
-      <c r="F78" s="6" t="inlineStr">
+      <c r="F78" t="inlineStr">
         <is>
           <t>Focuses on design and maintenance of marine propulsion systems. Develops expertise in mechanical and marine systems engineering. Focuses on ship engine performance. Graduates work in shipping, engineering, and maritime industries.</t>
         </is>
       </c>
-      <c r="G78" s="6" t="n"/>
-      <c r="H78" s="6" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="6" t="inlineStr">
+      <c r="A79" t="inlineStr">
         <is>
           <t>PhD in Marketing and Entrepreneurship</t>
         </is>
       </c>
-      <c r="B79" s="6" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>DEG-000078</t>
         </is>
       </c>
-      <c r="C79" s="6" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D79" s="6" t="inlineStr">
+      <c r="D79" t="inlineStr">
         <is>
           <t>Entrepreneurship</t>
         </is>
       </c>
-      <c r="E79" s="6" t="n">
+      <c r="E79" t="n">
         <v>3</v>
       </c>
-      <c r="F79" s="6" t="inlineStr">
+      <c r="F79" t="inlineStr">
         <is>
           <t>Studies marketing strategies for new ventures and startups. Develops expertise in innovation, branding, and business development. Focuses on entrepreneurial growth. Graduates work in startups, consulting, and business development.</t>
         </is>
       </c>
-      <c r="G79" s="6" t="n"/>
-      <c r="H79" s="6" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="6" t="inlineStr">
+      <c r="A80" t="inlineStr">
         <is>
           <t>PhD in Phonetics and Phonology</t>
         </is>
       </c>
-      <c r="B80" s="6" t="inlineStr">
+      <c r="B80" t="inlineStr">
         <is>
           <t>DEG-000079</t>
         </is>
       </c>
-      <c r="C80" s="6" t="inlineStr">
+      <c r="C80" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D80" s="6" t="inlineStr">
+      <c r="D80" t="inlineStr">
         <is>
           <t>Linguistics</t>
         </is>
       </c>
-      <c r="E80" s="6" t="n">
+      <c r="E80" t="n">
         <v>3</v>
       </c>
-      <c r="F80" s="6" t="inlineStr">
+      <c r="F80" t="inlineStr">
         <is>
           <t>Combines speech sound analysis with language sound systems. Develops expertise in linguistic theory and speech research. Focuses on sound structure and communication. Graduates work in academia, linguistics, and speech technology.</t>
         </is>
       </c>
-      <c r="G80" s="6" t="n"/>
-      <c r="H80" s="6" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="6" t="inlineStr">
+      <c r="A81" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Nursing and Allied Health</t>
         </is>
       </c>
-      <c r="B81" s="6" t="inlineStr">
+      <c r="B81" t="inlineStr">
         <is>
           <t>DEG-000080</t>
         </is>
       </c>
-      <c r="C81" s="6" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D81" s="6" t="inlineStr">
+      <c r="D81" t="inlineStr">
         <is>
           <t>Nursing and Allied Health</t>
         </is>
       </c>
-      <c r="E81" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F81" s="6" t="inlineStr">
+      <c r="E81" t="n">
+        <v>2</v>
+      </c>
+      <c r="F81" t="inlineStr">
         <is>
           <t>Studies basic nursing and healthcare support. Develops clinical and patient care skills. Focuses on healthcare services. Prepares graduates for healthcare support roles.</t>
         </is>
       </c>
-      <c r="G81" s="6" t="n"/>
-      <c r="H81" s="6" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="6" t="inlineStr">
+      <c r="A82" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Medical Assistant</t>
         </is>
       </c>
-      <c r="B82" s="6" t="inlineStr">
+      <c r="B82" t="inlineStr">
         <is>
           <t>DEG-000081</t>
         </is>
       </c>
-      <c r="C82" s="6" t="inlineStr">
+      <c r="C82" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D82" s="6" t="inlineStr">
+      <c r="D82" t="inlineStr">
         <is>
           <t>Medical Assistance</t>
         </is>
       </c>
-      <c r="E82" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F82" s="6" t="inlineStr">
+      <c r="E82" t="n">
+        <v>2</v>
+      </c>
+      <c r="F82" t="inlineStr">
         <is>
           <t>Studies clinical and administrative healthcare support. Develops patient care skills. Focuses on medical office practice. Prepares graduates for healthcare support roles.</t>
         </is>
       </c>
-      <c r="G82" s="6" t="n"/>
-      <c r="H82" s="6" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="6" t="inlineStr">
+      <c r="A83" t="inlineStr">
         <is>
           <t>Associate of Science in Radiography</t>
         </is>
       </c>
-      <c r="B83" s="6" t="inlineStr">
+      <c r="B83" t="inlineStr">
         <is>
           <t>DEG-000082</t>
         </is>
       </c>
-      <c r="C83" s="6" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D83" s="6" t="inlineStr">
+      <c r="D83" t="inlineStr">
         <is>
           <t>Radiography</t>
         </is>
       </c>
-      <c r="E83" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F83" s="6" t="inlineStr">
+      <c r="E83" t="n">
+        <v>2</v>
+      </c>
+      <c r="F83" t="inlineStr">
         <is>
           <t>Studies medical imaging and radiographic techniques. Develops imaging, patient care, and technical skills. Focuses on diagnostic imaging procedures. Graduates work in hospitals and medical imaging departments.</t>
         </is>
       </c>
-      <c r="G83" s="6" t="n"/>
-      <c r="H83" s="6" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="6" t="inlineStr">
+      <c r="A84" t="inlineStr">
         <is>
           <t>Associate of Arts in Marketing</t>
         </is>
       </c>
-      <c r="B84" s="6" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>DEG-000083</t>
         </is>
       </c>
-      <c r="C84" s="6" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D84" s="6" t="inlineStr">
+      <c r="D84" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="E84" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F84" s="6" t="inlineStr">
+      <c r="E84" t="n">
+        <v>2</v>
+      </c>
+      <c r="F84" t="inlineStr">
         <is>
           <t>Studies marketing strategies and consumer behavior. Develops communication, analytical, and promotional skills. Focuses on branding, advertising, and market research. Graduates work in marketing, sales, and retail.</t>
         </is>
       </c>
-      <c r="G84" s="6" t="n"/>
-      <c r="H84" s="6" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="6" t="inlineStr">
+      <c r="A85" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Dental Hygiene</t>
         </is>
       </c>
-      <c r="B85" s="6" t="inlineStr">
+      <c r="B85" t="inlineStr">
         <is>
           <t>DEG-000084</t>
         </is>
       </c>
-      <c r="C85" s="6" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D85" s="6" t="inlineStr">
+      <c r="D85" t="inlineStr">
         <is>
           <t>Dental Hygiene</t>
         </is>
       </c>
-      <c r="E85" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F85" s="6" t="inlineStr">
+      <c r="E85" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" t="inlineStr">
         <is>
           <t>Studies preventive dental care and oral health. Develops clinical, patient care, and communication skills. Focuses on dental hygiene procedures and education. Graduates work in dental clinics and healthcare facilities.</t>
         </is>
       </c>
-      <c r="G85" s="6" t="n"/>
-      <c r="H85" s="6" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="6" t="inlineStr">
+      <c r="A86" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Radiography</t>
         </is>
       </c>
-      <c r="B86" s="6" t="inlineStr">
+      <c r="B86" t="inlineStr">
         <is>
           <t>DEG-000085</t>
         </is>
       </c>
-      <c r="C86" s="6" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D86" s="6" t="inlineStr">
+      <c r="D86" t="inlineStr">
         <is>
           <t>Radiography</t>
         </is>
       </c>
-      <c r="E86" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F86" s="6" t="inlineStr">
+      <c r="E86" t="n">
+        <v>2</v>
+      </c>
+      <c r="F86" t="inlineStr">
         <is>
           <t>Studies diagnostic imaging and radiographic procedures. Develops imaging, patient care, and technical skills. Focuses on producing medical images for diagnosis. Graduates work in hospitals and diagnostic imaging centers.</t>
         </is>
       </c>
-      <c r="G86" s="6" t="n"/>
-      <c r="H86" s="6" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="6" t="inlineStr">
+      <c r="A87" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Diagnostic Medical Sonography</t>
         </is>
       </c>
-      <c r="B87" s="6" t="inlineStr">
+      <c r="B87" t="inlineStr">
         <is>
           <t>DEG-000086</t>
         </is>
       </c>
-      <c r="C87" s="6" t="inlineStr">
+      <c r="C87" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D87" s="6" t="inlineStr">
+      <c r="D87" t="inlineStr">
         <is>
           <t>Diagnostic Medical Sonography</t>
         </is>
       </c>
-      <c r="E87" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F87" s="6" t="inlineStr">
+      <c r="E87" t="n">
+        <v>2</v>
+      </c>
+      <c r="F87" t="inlineStr">
         <is>
           <t>Studies ultrasound imaging and patient care. Develops diagnostic imaging, technical, and clinical skills. Focuses on safe and accurate medical sonography. Prepares graduates for careers as diagnostic medical sonographers.</t>
         </is>
       </c>
-      <c r="G87" s="6" t="n"/>
-      <c r="H87" s="6" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="6" t="inlineStr">
+      <c r="A88" t="inlineStr">
         <is>
           <t>Associate of Science in Music Production</t>
         </is>
       </c>
-      <c r="B88" s="6" t="inlineStr">
+      <c r="B88" t="inlineStr">
         <is>
           <t>DEG-000087</t>
         </is>
       </c>
-      <c r="C88" s="6" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D88" s="6" t="inlineStr">
+      <c r="D88" t="inlineStr">
         <is>
           <t>Music Production</t>
         </is>
       </c>
-      <c r="E88" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F88" s="6" t="inlineStr">
+      <c r="E88" t="n">
+        <v>2</v>
+      </c>
+      <c r="F88" t="inlineStr">
         <is>
           <t>Studies audio recording, music technology, and production. Develops recording, editing, and sound design skills. Focuses on creating professional music productions. Graduates work in recording studios and media production.</t>
         </is>
       </c>
-      <c r="G88" s="6" t="n"/>
-      <c r="H88" s="6" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="6" t="inlineStr">
+      <c r="A89" t="inlineStr">
         <is>
           <t>Associate of Applied Science</t>
         </is>
       </c>
-      <c r="B89" s="6" t="inlineStr">
+      <c r="B89" t="inlineStr">
         <is>
           <t>DEG-000088</t>
         </is>
       </c>
-      <c r="C89" s="6" t="inlineStr">
+      <c r="C89" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D89" s="6" t="inlineStr">
+      <c r="D89" t="inlineStr">
         <is>
           <t>Applied Science</t>
         </is>
       </c>
-      <c r="E89" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F89" s="6" t="inlineStr">
+      <c r="E89" t="n">
+        <v>2</v>
+      </c>
+      <c r="F89" t="inlineStr">
         <is>
           <t>Studies practical scientific and technical applications. Develops laboratory, technical, and problem-solving skills. Focuses on career-ready scientific knowledge. Graduates work in technical, healthcare, and industrial roles.</t>
         </is>
       </c>
-      <c r="G89" s="6" t="n"/>
-      <c r="H89" s="6" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="6" t="inlineStr">
+      <c r="A90" t="inlineStr">
         <is>
           <t>Associate of Science in Nursing</t>
         </is>
       </c>
-      <c r="B90" s="6" t="inlineStr">
+      <c r="B90" t="inlineStr">
         <is>
           <t>DEG-000089</t>
         </is>
       </c>
-      <c r="C90" s="6" t="inlineStr">
+      <c r="C90" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D90" s="6" t="inlineStr">
+      <c r="D90" t="inlineStr">
         <is>
           <t>Nursing</t>
         </is>
       </c>
-      <c r="E90" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F90" s="6" t="inlineStr">
+      <c r="E90" t="n">
+        <v>2</v>
+      </c>
+      <c r="F90" t="inlineStr">
         <is>
           <t>Studies nursing science and patient-centered care. Develops clinical, communication, and healthcare skills. Focuses on safe nursing practice and health promotion. Graduates work in hospitals, clinics, and healthcare facilities.</t>
         </is>
       </c>
-      <c r="G90" s="6" t="n"/>
-      <c r="H90" s="6" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="6" t="inlineStr">
+      <c r="A91" t="inlineStr">
         <is>
           <t>Associate of Arts</t>
         </is>
       </c>
-      <c r="B91" s="6" t="inlineStr">
+      <c r="B91" t="inlineStr">
         <is>
           <t>DEG-000090</t>
         </is>
       </c>
-      <c r="C91" s="6" t="inlineStr">
+      <c r="C91" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D91" s="6" t="inlineStr">
+      <c r="D91" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="E91" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F91" s="6" t="inlineStr">
+      <c r="E91" t="n">
+        <v>2</v>
+      </c>
+      <c r="F91" t="inlineStr">
         <is>
           <t>Studies humanities, social sciences, and communication. Develops critical thinking, writing, and analytical skills. Focuses on broad academic preparation. Graduates continue higher education or enter diverse professional fields.</t>
         </is>
       </c>
-      <c r="G91" s="6" t="n"/>
-      <c r="H91" s="6" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="6" t="inlineStr">
+      <c r="A92" t="inlineStr">
         <is>
           <t>Associate of Arts Degree</t>
         </is>
       </c>
-      <c r="B92" s="6" t="inlineStr">
+      <c r="B92" t="inlineStr">
         <is>
           <t>DEG-000091</t>
         </is>
       </c>
-      <c r="C92" s="6" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D92" s="6" t="inlineStr">
+      <c r="D92" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="E92" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F92" s="6" t="inlineStr">
+      <c r="E92" t="n">
+        <v>2</v>
+      </c>
+      <c r="F92" t="inlineStr">
         <is>
           <t>Studies a broad range of humanities and social sciences. Develops communication, research, and critical thinking skills. Focuses on transferable academic knowledge. Graduates continue higher education or pursue entry-level careers.</t>
         </is>
       </c>
-      <c r="G92" s="6" t="n"/>
-      <c r="H92" s="6" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="6" t="inlineStr">
+      <c r="A93" t="inlineStr">
         <is>
           <t>Associate of Nursing</t>
         </is>
       </c>
-      <c r="B93" s="6" t="inlineStr">
+      <c r="B93" t="inlineStr">
         <is>
           <t>DEG-000092</t>
         </is>
       </c>
-      <c r="C93" s="6" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D93" s="6" t="inlineStr">
+      <c r="D93" t="inlineStr">
         <is>
           <t>Nursing</t>
         </is>
       </c>
-      <c r="E93" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F93" s="6" t="inlineStr">
+      <c r="E93" t="n">
+        <v>2</v>
+      </c>
+      <c r="F93" t="inlineStr">
         <is>
           <t>Studies patient care and foundational nursing practice. Develops clinical, communication, and healthcare skills. Focuses on evidence-based nursing and patient safety. Graduates work in hospitals, clinics, and healthcare facilities.</t>
         </is>
       </c>
-      <c r="G93" s="6" t="n"/>
-      <c r="H93" s="6" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="6" t="inlineStr">
+      <c r="A94" t="inlineStr">
         <is>
           <t>Associate of Science in Business</t>
         </is>
       </c>
-      <c r="B94" s="6" t="inlineStr">
+      <c r="B94" t="inlineStr">
         <is>
           <t>DEG-000093</t>
         </is>
       </c>
-      <c r="C94" s="6" t="inlineStr">
+      <c r="C94" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D94" s="6" t="inlineStr">
+      <c r="D94" t="inlineStr">
         <is>
           <t>Business</t>
         </is>
       </c>
-      <c r="E94" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F94" s="6" t="inlineStr">
+      <c r="E94" t="n">
+        <v>2</v>
+      </c>
+      <c r="F94" t="inlineStr">
         <is>
           <t>Studies core business principles and organizational practices. Develops communication, management, and analytical skills. Focuses on finance, marketing, and operations. Graduates work in business support, retail, and administration.</t>
         </is>
       </c>
-      <c r="G94" s="6" t="n"/>
-      <c r="H94" s="6" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="6" t="inlineStr">
+      <c r="A95" t="inlineStr">
         <is>
           <t>Associate of Science</t>
         </is>
       </c>
-      <c r="B95" s="6" t="inlineStr">
+      <c r="B95" t="inlineStr">
         <is>
           <t>DEG-000094</t>
         </is>
       </c>
-      <c r="C95" s="6" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D95" s="6" t="inlineStr">
+      <c r="D95" t="inlineStr">
         <is>
           <t>Science</t>
         </is>
       </c>
-      <c r="E95" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F95" s="6" t="inlineStr">
+      <c r="E95" t="n">
+        <v>2</v>
+      </c>
+      <c r="F95" t="inlineStr">
         <is>
           <t>Studies foundational scientific concepts and methods. Develops laboratory, analytical, and problem-solving skills. Focuses on biology, chemistry, and scientific inquiry. Graduates continue science studies or work in technical fields.</t>
         </is>
       </c>
-      <c r="G95" s="6" t="n"/>
-      <c r="H95" s="6" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="6" t="inlineStr">
+      <c r="A96" t="inlineStr">
         <is>
           <t>Associate of Science in Business Administration</t>
         </is>
       </c>
-      <c r="B96" s="6" t="inlineStr">
+      <c r="B96" t="inlineStr">
         <is>
           <t>DEG-000095</t>
         </is>
       </c>
-      <c r="C96" s="6" t="inlineStr">
+      <c r="C96" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D96" s="6" t="inlineStr">
+      <c r="D96" t="inlineStr">
         <is>
           <t>Business Administration</t>
         </is>
       </c>
-      <c r="E96" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F96" s="6" t="inlineStr">
+      <c r="E96" t="n">
+        <v>2</v>
+      </c>
+      <c r="F96" t="inlineStr">
         <is>
           <t>Studies business operations and management fundamentals. Develops organizational, communication, and leadership skills. Focuses on business strategy and workplace effectiveness. Graduates work in administration, sales, and operations.</t>
         </is>
       </c>
-      <c r="G96" s="6" t="n"/>
-      <c r="H96" s="6" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="6" t="inlineStr">
+      <c r="A97" t="inlineStr">
         <is>
           <t>Associate of Science in Biology and Ecology</t>
         </is>
       </c>
-      <c r="B97" s="6" t="inlineStr">
+      <c r="B97" t="inlineStr">
         <is>
           <t>DEG-000096</t>
         </is>
       </c>
-      <c r="C97" s="6" t="inlineStr">
+      <c r="C97" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D97" s="6" t="inlineStr">
+      <c r="D97" t="inlineStr">
         <is>
           <t>Biology and Ecology</t>
         </is>
       </c>
-      <c r="E97" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F97" s="6" t="inlineStr">
+      <c r="E97" t="n">
+        <v>2</v>
+      </c>
+      <c r="F97" t="inlineStr">
         <is>
           <t>Studies biological systems and ecological processes. Develops laboratory, fieldwork, and analytical skills. Focuses on ecosystems, biodiversity, and environmental science. Graduates work in environmental organizations and laboratories.</t>
         </is>
       </c>
-      <c r="G97" s="6" t="n"/>
-      <c r="H97" s="6" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="6" t="inlineStr">
+      <c r="A98" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Accounting</t>
         </is>
       </c>
-      <c r="B98" s="6" t="inlineStr">
+      <c r="B98" t="inlineStr">
         <is>
           <t>DEG-000097</t>
         </is>
       </c>
-      <c r="C98" s="6" t="inlineStr">
+      <c r="C98" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D98" s="6" t="inlineStr">
+      <c r="D98" t="inlineStr">
         <is>
           <t>Accounting</t>
         </is>
       </c>
-      <c r="E98" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F98" s="6" t="inlineStr">
+      <c r="E98" t="n">
+        <v>2</v>
+      </c>
+      <c r="F98" t="inlineStr">
         <is>
           <t>Studies accounting principles and financial reporting. Develops bookkeeping, financial analysis, and accounting software skills. Focuses on business finance and compliance. Graduates work in accounting, bookkeeping, and finance support.</t>
         </is>
       </c>
-      <c r="G98" s="6" t="n"/>
-      <c r="H98" s="6" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="6" t="inlineStr">
+      <c r="A99" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Hospitality Management</t>
         </is>
       </c>
-      <c r="B99" s="6" t="inlineStr">
+      <c r="B99" t="inlineStr">
         <is>
           <t>DEG-000098</t>
         </is>
       </c>
-      <c r="C99" s="6" t="inlineStr">
+      <c r="C99" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D99" s="6" t="inlineStr">
+      <c r="D99" t="inlineStr">
         <is>
           <t>Hospitality Management</t>
         </is>
       </c>
-      <c r="E99" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F99" s="6" t="inlineStr">
+      <c r="E99" t="n">
+        <v>2</v>
+      </c>
+      <c r="F99" t="inlineStr">
         <is>
           <t>Studies hospitality operations and customer service management. Develops leadership, communication, and operational skills. Focuses on hotels, tourism, and guest satisfaction. Graduates work in hospitality, tourism, and hotel management.</t>
         </is>
       </c>
-      <c r="G99" s="6" t="n"/>
-      <c r="H99" s="6" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="6" t="inlineStr">
+      <c r="A100" t="inlineStr">
         <is>
           <t>Associate of Science in Computer Science</t>
         </is>
       </c>
-      <c r="B100" s="6" t="inlineStr">
+      <c r="B100" t="inlineStr">
         <is>
           <t>DEG-000099</t>
         </is>
       </c>
-      <c r="C100" s="6" t="inlineStr">
+      <c r="C100" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D100" s="6" t="inlineStr">
+      <c r="D100" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="E100" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F100" s="6" t="inlineStr">
+      <c r="E100" t="n">
+        <v>2</v>
+      </c>
+      <c r="F100" t="inlineStr">
         <is>
           <t>Studies computing principles and software development. Develops programming, analytical, and technical problem-solving skills. Focuses on algorithms, databases, and computer systems. Graduates work in IT support and software development.</t>
         </is>
       </c>
-      <c r="G100" s="6" t="n"/>
-      <c r="H100" s="6" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="6" t="inlineStr">
+      <c r="A101" t="inlineStr">
         <is>
           <t>Associate of Arts in Business Administration</t>
         </is>
       </c>
-      <c r="B101" s="6" t="inlineStr">
+      <c r="B101" t="inlineStr">
         <is>
           <t>DEG-000100</t>
         </is>
       </c>
-      <c r="C101" s="6" t="inlineStr">
+      <c r="C101" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D101" s="6" t="inlineStr">
+      <c r="D101" t="inlineStr">
         <is>
           <t>Business Administration</t>
         </is>
       </c>
-      <c r="E101" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F101" s="6" t="inlineStr">
+      <c r="E101" t="n">
+        <v>2</v>
+      </c>
+      <c r="F101" t="inlineStr">
         <is>
           <t>Studies business operations and organizational management. Develops leadership, communication, and administrative skills. Focuses on finance, marketing, and business practices. Graduates work in administration, retail, and business support.</t>
         </is>
       </c>
-      <c r="G101" s="6" t="n"/>
-      <c r="H101" s="6" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1" password="DB2D"/>

</xml_diff>

<commit_message>
Refresh Excel import templates for EmployeeCountRange.CLASSIFIED
Reran generate_excel_templates.py --protect-existing so organizations.xlsx's
numberOfEmployees dropdown picks up the new CLASSIFIED enum value from
schema.prisma. All existing data preserved (verified row counts and sample
cell values unchanged across all 11 templates) since --protect-existing
refreshes validation/dropdowns in place without touching cell values.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/api/data/excel_templates/degrees.xlsx
+++ b/apps/api/data/excel_templates/degrees.xlsx
@@ -57,7 +57,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
@@ -70,6 +70,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -491,3004 +494,3204 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Master in Philosophy and English Literature</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>DEG-000001</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Literature &amp; Philosophy</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="E2" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Focuses on literary and philosophical texts. Develops analytical and interpretive skills. Studies cultural theory. Emphasises critical reading. Prepares for academic careers.</t>
         </is>
       </c>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="6" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Master in Philosophy and Mathematics</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>DEG-000002</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Mathematical Philosophy</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" t="inlineStr">
+      <c r="E3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Focuses on logic and mathematical reasoning. Develops analytical and abstract thinking. Studies formal systems. Emphasises theoretical inquiry. Prepares for research careers.</t>
         </is>
       </c>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Master in Philosophy and Public Policy</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>DEG-000003</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Policy Studies</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" t="inlineStr">
+      <c r="E4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Focuses on ethical foundations of policy-making. Develops analytical and governance skills. Studies public systems. Emphasises decision frameworks. Prepares for policy roles.</t>
         </is>
       </c>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Master in Philosophy and Religion</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>DEG-000004</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Religious Studies</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" t="inlineStr">
+      <c r="E5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Focuses on philosophical analysis of religion. Develops interpretive and critical skills. Studies belief systems. Emphasises theological inquiry. Prepares for academic roles.</t>
         </is>
       </c>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Master in Photonics</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>DEG-000005</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Physics &amp; Engineering</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F6" t="inlineStr">
+      <c r="E6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Focuses on light manipulation and optical systems. Develops experimental and theoretical skills. Studies wave optics. Emphasises applied physics. Prepares for research roles.</t>
         </is>
       </c>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Master in Photonics and Quantum Sciences</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>DEG-000006</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Quantum Technology</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F7" t="inlineStr">
+      <c r="E7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Focuses on quantum optics and photonics. Develops theoretical and experimental skills. Studies quantum systems. Emphasises advanced research. Prepares for scientific careers.</t>
         </is>
       </c>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Master in Physical Sciences</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>DEG-000007</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Natural Sciences</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F8" t="inlineStr">
+      <c r="E8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Focuses on physics and related sciences. Develops analytical and experimental skills. Studies matter and energy. Emphasises research methods. Prepares for scientific careers.</t>
         </is>
       </c>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Master in Physical Therapy and Rehabilitation</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>DEG-000008</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Rehabilitation Science</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v>2</v>
-      </c>
-      <c r="F9" t="inlineStr">
+      <c r="E9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Focuses on restoring physical function after injury. Develops therapeutic skills. Studies movement recovery. Emphasises clinical rehabilitation. Prepares for therapy careers.</t>
         </is>
       </c>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Master in Physics and Technology of Nanostructures</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>DEG-000009</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Nanotechnology</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>2</v>
-      </c>
-      <c r="F10" t="inlineStr">
+      <c r="E10" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Focuses on engineered nanoscale structures. Develops experimental and fabrication skills. Studies quantum effects. Emphasises advanced materials. Prepares for research roles.</t>
         </is>
       </c>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Master in Physics and Thermal Physics of Innovative Nuclear Power Installations</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>DEG-000010</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Nuclear Energy</t>
         </is>
       </c>
-      <c r="E11" t="n">
-        <v>2</v>
-      </c>
-      <c r="F11" t="inlineStr">
+      <c r="E11" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Focuses on thermal and reactor physics. Develops modelling and engineering skills. Studies nuclear systems. Emphasises energy innovation. Prepares for nuclear industry roles.</t>
         </is>
       </c>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Master in Physics of Complex Systems and Biophysics</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>DEG-000011</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Biophysics</t>
         </is>
       </c>
-      <c r="E12" t="n">
-        <v>2</v>
-      </c>
-      <c r="F12" t="inlineStr">
+      <c r="E12" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Focuses on complex systems in biology and physics. Develops analytical skills. Studies living systems. Emphasises interdisciplinary research. Prepares for scientific careers.</t>
         </is>
       </c>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Master in Physics with Mathematics</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>DEG-000012</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Mathematical Physics</t>
         </is>
       </c>
-      <c r="E13" t="n">
-        <v>2</v>
-      </c>
-      <c r="F13" t="inlineStr">
+      <c r="E13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Focuses on mathematical methods in physics. Develops modelling and analytical skills. Studies theoretical frameworks. Emphasises problem-solving. Prepares for research roles.</t>
         </is>
       </c>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Master in Physics with Planetary and Space Physics</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>DEG-000013</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Space Physics</t>
         </is>
       </c>
-      <c r="E14" t="n">
-        <v>2</v>
-      </c>
-      <c r="F14" t="inlineStr">
+      <c r="E14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Focuses on planetary systems and space environments. Develops analytical skills. Studies solar and planetary physics. Emphasises space science. Prepares for research careers.</t>
         </is>
       </c>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Master in Planning and Management of Tourism Systems</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>DEG-000014</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Tourism Management</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>2</v>
-      </c>
-      <c r="F15" t="inlineStr">
+      <c r="E15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Focuses on tourism system design and management. Develops planning and business skills. Studies tourism flows. Emphasises sustainability. Prepares for tourism industry roles.</t>
         </is>
       </c>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Master in Plasma Physics, Spectroscopy and Self-Organization</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>DEG-000015</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Applied Physics</t>
         </is>
       </c>
-      <c r="E16" t="n">
-        <v>2</v>
-      </c>
-      <c r="F16" t="inlineStr">
+      <c r="E16" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Focuses on plasma diagnostics and systems behaviour. Develops analytical skills. Studies light-matter interaction. Emphasises advanced research. Prepares for physics careers.</t>
         </is>
       </c>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Master in Play Therapy</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>DEG-000016</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>Psychotherapy</t>
         </is>
       </c>
-      <c r="E17" t="n">
-        <v>2</v>
-      </c>
-      <c r="F17" t="inlineStr">
+      <c r="E17" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>Focuses on therapeutic use of play for children. Develops counselling skills. Studies child psychology. Emphasises emotional development. Prepares for clinical therapy roles.</t>
         </is>
       </c>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Master in Podiatric Surgery</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>DEG-000017</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>Surgical Medicine</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>2</v>
-      </c>
-      <c r="F18" t="inlineStr">
+      <c r="E18" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>Focuses on surgical treatment of foot disorders. Develops clinical and surgical skills. Studies anatomy and pathology. Emphasises operative care. Prepares for surgical roles.</t>
         </is>
       </c>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Master in Portuguese and Business</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>DEG-000018</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>Business Communication</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F19" t="inlineStr">
+      <c r="E19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>Focuses on Portuguese language in business contexts. Develops communication skills. Studies commerce and culture. Emphasises international trade. Prepares for business roles.</t>
         </is>
       </c>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Master in Post-production with Sound Design</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>DEG-000019</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>Media Production</t>
         </is>
       </c>
-      <c r="E20" t="n">
-        <v>2</v>
-      </c>
-      <c r="F20" t="inlineStr">
+      <c r="E20" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>Focuses on audio post-production for media. Develops technical and creative skills. Studies sound design. Emphasises film and media industries. Prepares for production roles.</t>
         </is>
       </c>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Master in Power, Electronic and Telecommunication Engineering</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>DEG-000020</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>Electrical Engineering</t>
         </is>
       </c>
-      <c r="E21" t="n">
-        <v>2</v>
-      </c>
-      <c r="F21" t="inlineStr">
+      <c r="E21" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>Focuses on integrated power and communication systems. Develops technical skills. Studies networks and electronics. Emphasises infrastructure. Prepares for engineering roles.</t>
         </is>
       </c>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>Master in Process Engineering</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>DEG-000021</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>Chemical/Industrial Engineering</t>
         </is>
       </c>
-      <c r="E22" t="n">
-        <v>2</v>
-      </c>
-      <c r="F22" t="inlineStr">
+      <c r="E22" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>Focuses on industrial process design and optimisation. Develops engineering skills. Studies production systems. Emphasises efficiency and safety. Prepares for industry roles.</t>
         </is>
       </c>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Master in Professional Archaeology and Comprehensive Heritage Management</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>DEG-000022</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>Archaeology</t>
         </is>
       </c>
-      <c r="E23" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" t="inlineStr">
+      <c r="E23" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>Focuses on archaeological practice and heritage management. Develops field skills. Studies cultural preservation. Emphasises applied archaeology. Prepares for heritage roles.</t>
         </is>
       </c>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Master in Professional Non-surgical Aesthetic Practice</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>DEG-000023</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>Aesthetic Medicine</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>2</v>
-      </c>
-      <c r="F24" t="inlineStr">
+      <c r="E24" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>Focuses on cosmetic non-surgical treatments. Develops clinical and procedural skills. Studies skin aesthetics. Emphasises patient care. Prepares for aesthetic practice roles.</t>
         </is>
       </c>
+      <c r="G24" s="6" t="n"/>
+      <c r="H24" s="6" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Master in Professional Studies in Education</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>DEG-000024</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E25" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" t="inlineStr">
+      <c r="E25" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>Focuses on advanced teaching and learning practice. Develops pedagogical skills. Studies education systems. Emphasises instructional improvement. Prepares for educator roles.</t>
         </is>
       </c>
+      <c r="G25" s="6" t="n"/>
+      <c r="H25" s="6" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Master in Professional Translation Studies</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>DEG-000025</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>Translation Studies</t>
         </is>
       </c>
-      <c r="E26" t="n">
-        <v>2</v>
-      </c>
-      <c r="F26" t="inlineStr">
+      <c r="E26" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>Focuses on advanced translation theory and practice. Develops language skills. Studies translation techniques. Emphasises accuracy and fluency. Prepares for translator roles.</t>
         </is>
       </c>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="6" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>Master in Prostate Cancer Care</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>DEG-000026</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>Oncology</t>
         </is>
       </c>
-      <c r="E27" t="n">
-        <v>2</v>
-      </c>
-      <c r="F27" t="inlineStr">
+      <c r="E27" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>Focuses on diagnosis and treatment of prostate cancer. Develops clinical skills. Studies oncology care pathways. Emphasises patient management. Prepares for healthcare roles.</t>
         </is>
       </c>
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="6" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>Master in Psychology Conversion</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>DEG-000027</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>Conversion Psychology</t>
         </is>
       </c>
-      <c r="E28" t="n">
-        <v>2</v>
-      </c>
-      <c r="F28" t="inlineStr">
+      <c r="E28" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>Focuses on foundational psychology training. Develops core analytical skills. Studies psychological theory. Emphasises transition into field. Prepares for psychology careers.</t>
         </is>
       </c>
+      <c r="G28" s="6" t="n"/>
+      <c r="H28" s="6" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>Master in Psycho-oncology and Palliative Care</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>DEG-000028</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>Health Psychology</t>
         </is>
       </c>
-      <c r="E29" t="n">
-        <v>2</v>
-      </c>
-      <c r="F29" t="inlineStr">
+      <c r="E29" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>Focuses on psychological support in cancer care. Develops clinical intervention skills. Studies patient wellbeing. Emphasises end-of-life care. Prepares for healthcare roles.</t>
         </is>
       </c>
+      <c r="G29" s="6" t="n"/>
+      <c r="H29" s="6" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Master in Public Health, Public Health Nutrition and Epidemiology</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>DEG-000029</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>Master</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>Public Health Nutrition</t>
         </is>
       </c>
-      <c r="E30" t="n">
-        <v>2</v>
-      </c>
-      <c r="F30" t="inlineStr">
+      <c r="E30" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>Focuses on nutrition and disease prevention. Develops epidemiological skills. Studies diet and population health. Emphasises prevention strategies. Prepares for health roles.</t>
         </is>
       </c>
+      <c r="G30" s="6" t="n"/>
+      <c r="H30" s="6" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Design in Visual Communication and BA in International Studies</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>DEG-000030</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>Design / Communication</t>
         </is>
       </c>
-      <c r="E31" t="n">
+      <c r="E31" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>Combines visual communication with global studies. Covers branding and media. Develops creative skills. Prepares for design careers.</t>
         </is>
       </c>
+      <c r="G31" s="6" t="n"/>
+      <c r="H31" s="6" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Teaching and BA in Mathematics</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>DEG-000031</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>Education / Mathematics</t>
         </is>
       </c>
-      <c r="E32" t="n">
+      <c r="E32" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>Combines teaching with mathematics. Covers pedagogy and quantitative skills. Develops instructional ability. Prepares for teaching roles.</t>
         </is>
       </c>
+      <c r="G32" s="6" t="n"/>
+      <c r="H32" s="6" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Health Science in Traditional Chinese Medicine and BA in International Studies</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>DEG-000032</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>Health / Traditional Medicine</t>
         </is>
       </c>
-      <c r="E33" t="n">
+      <c r="E33" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <t>Combines Chinese medicine with global studies. Covers holistic health systems. Develops clinical knowledge. Prepares for healthcare roles.</t>
         </is>
       </c>
+      <c r="G33" s="6" t="n"/>
+      <c r="H33" s="6" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Teaching and BA in Visual Arts</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>DEG-000033</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>Education / Arts</t>
         </is>
       </c>
-      <c r="E34" t="n">
+      <c r="E34" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="6" t="inlineStr">
         <is>
           <t>Combines teaching with visual arts practice. Covers pedagogy and creativity. Develops instructional skills. Prepares for arts education roles.</t>
         </is>
       </c>
+      <c r="G34" s="6" t="n"/>
+      <c r="H34" s="6" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Education and BA in International Studies</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>DEG-000034</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E35" t="n">
+      <c r="E35" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
         <is>
           <t>Combines teaching qualifications with global studies. Covers pedagogy and culture. Develops instructional skills. Prepares for education roles.</t>
         </is>
       </c>
+      <c r="G35" s="6" t="n"/>
+      <c r="H35" s="6" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Teaching and BA in Technology</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>DEG-000035</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>Education / Technology</t>
         </is>
       </c>
-      <c r="E36" t="n">
+      <c r="E36" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="6" t="inlineStr">
         <is>
           <t>Combines teaching with technology studies. Covers digital tools and pedagogy. Develops instructional skills. Prepares for STEM education roles.</t>
         </is>
       </c>
+      <c r="G36" s="6" t="n"/>
+      <c r="H36" s="6" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Journalism and Professional Writing and BA in Creative Writing and Literature</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>DEG-000036</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>Journalism / Writing</t>
         </is>
       </c>
-      <c r="E37" t="n">
+      <c r="E37" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
         <is>
           <t>Combines journalism with creative writing. Covers reporting, storytelling, and media. Develops communication skills. Prepares for media careers.</t>
         </is>
       </c>
+      <c r="G37" s="6" t="n"/>
+      <c r="H37" s="6" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Commerce, BA in Psychology</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>DEG-000037</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>Business / Psychology</t>
         </is>
       </c>
-      <c r="E38" t="n">
+      <c r="E38" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>Combines commerce with psychology studies. Covers business strategy and human behaviour. Develops analytical skills. Prepares for corporate roles.</t>
         </is>
       </c>
+      <c r="G38" s="6" t="n"/>
+      <c r="H38" s="6" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Nursing and BA in International Studies</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>DEG-000038</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>Nursing</t>
         </is>
       </c>
-      <c r="E39" t="n">
+      <c r="E39" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>Combines nursing practice with global studies. Covers healthcare systems and patient care. Develops clinical skills. Prepares for nursing careers.</t>
         </is>
       </c>
+      <c r="G39" s="6" t="n"/>
+      <c r="H39" s="6" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Teaching and BA in Humanities</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>DEG-000039</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E40" t="n">
+      <c r="E40" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>Combines teaching qualification with humanities studies. Covers pedagogy and culture. Develops instructional skills. Prepares for education roles.</t>
         </is>
       </c>
+      <c r="G40" s="6" t="n"/>
+      <c r="H40" s="6" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Design in Interior Architecture and BA in International Studies</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>DEG-000040</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>Design / Architecture</t>
         </is>
       </c>
-      <c r="E41" t="n">
+      <c r="E41" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="6" t="inlineStr">
         <is>
           <t>Combines interior design with global studies. Covers spatial design and culture. Develops creative and technical skills. Prepares for design careers.</t>
         </is>
       </c>
+      <c r="G41" s="6" t="n"/>
+      <c r="H41" s="6" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Design in Product Design and BA in International Studies</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>DEG-000041</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>Design / Product</t>
         </is>
       </c>
-      <c r="E42" t="n">
+      <c r="E42" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="6" t="inlineStr">
         <is>
           <t>Combines product design with global studies. Covers innovation and user-centred design. Develops technical skills. Prepares for design industry roles.</t>
         </is>
       </c>
+      <c r="G42" s="6" t="n"/>
+      <c r="H42" s="6" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Medical Science and BA in International Studies</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>DEG-000042</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>Medical Science</t>
         </is>
       </c>
-      <c r="E43" t="n">
+      <c r="E43" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="6" t="inlineStr">
         <is>
           <t>Combines medical science with global studies. Covers biology, health systems, and policy. Develops scientific skills. Prepares for health sector roles.</t>
         </is>
       </c>
+      <c r="G43" s="6" t="n"/>
+      <c r="H43" s="6" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Design in Animation and BA in International Studies</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>DEG-000043</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>Design / International Studies</t>
         </is>
       </c>
-      <c r="E44" t="n">
+      <c r="E44" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="6" t="inlineStr">
         <is>
           <t>Combines animation with global cultural studies. Covers storytelling and media production. Develops creative skills. Prepares for animation and media roles.</t>
         </is>
       </c>
+      <c r="G44" s="6" t="n"/>
+      <c r="H44" s="6" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Design in Photography and BA in International Studies</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>DEG-000044</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>Design / Photography</t>
         </is>
       </c>
-      <c r="E45" t="n">
+      <c r="E45" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <t>Combines photography with international studies. Covers visual storytelling and culture. Develops artistic skills. Prepares for media and photography roles.</t>
         </is>
       </c>
+      <c r="G45" s="6" t="n"/>
+      <c r="H45" s="6" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Commerce and BA in Psychology and Economics</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>DEG-000045</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>Business / Social Science</t>
         </is>
       </c>
-      <c r="E46" t="n">
+      <c r="E46" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="6" t="inlineStr">
         <is>
           <t>Integrates commerce, psychology, and economics. Covers markets, behaviour, and policy. Develops analytical skills. Prepares for finance and consulting roles.</t>
         </is>
       </c>
+      <c r="G46" s="6" t="n"/>
+      <c r="H46" s="6" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Communication in Creative Writing and BA in International Studies</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>DEG-000046</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>Communication / International Studies</t>
         </is>
       </c>
-      <c r="E47" t="n">
+      <c r="E47" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="6" t="inlineStr">
         <is>
           <t>Combines creative writing with global studies. Covers media, culture, and communication. Develops storytelling skills. Prepares for media and international roles.</t>
         </is>
       </c>
+      <c r="G47" s="6" t="n"/>
+      <c r="H47" s="6" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Construction Project Management, BA in International Studies</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>DEG-000047</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
         <is>
           <t>Construction / International Studies</t>
         </is>
       </c>
-      <c r="E48" t="n">
+      <c r="E48" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="6" t="inlineStr">
         <is>
           <t>Combines construction management with global studies. Covers planning, infrastructure, and policy. Develops leadership skills. Prepares for project management roles.</t>
         </is>
       </c>
+      <c r="G48" s="6" t="n"/>
+      <c r="H48" s="6" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Commerce and BA in Psychology</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>DEG-000048</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>Business / Psychology</t>
         </is>
       </c>
-      <c r="E49" t="n">
+      <c r="E49" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F49" s="6" t="inlineStr">
         <is>
           <t>Combines business commerce with psychological science. Covers markets, behaviour, and analytics. Develops interdisciplinary skills. Prepares for business and HR roles.</t>
         </is>
       </c>
+      <c r="G49" s="6" t="n"/>
+      <c r="H49" s="6" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>Bachelor in Transfer Degree</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t>DEG-000049</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t>General Studies</t>
         </is>
       </c>
-      <c r="E50" t="n">
+      <c r="E50" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F50" s="6" t="inlineStr">
         <is>
           <t>Provides foundational academic coursework for transfer. Develops core academic skills. Focuses on university progression pathways. Prepares students for advanced degrees.</t>
         </is>
       </c>
+      <c r="G50" s="6" t="n"/>
+      <c r="H50" s="6" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="6" t="inlineStr">
         <is>
           <t>Bachelor and MBA in Supply Chain Management</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t>DEG-000050</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>Business / Logistics</t>
         </is>
       </c>
-      <c r="E51" t="n">
+      <c r="E51" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F51" s="6" t="inlineStr">
         <is>
           <t>Integrated program covering supply chain and advanced business management. Covers logistics, operations, and strategy. Develops leadership skills. Prepares for senior management roles.</t>
         </is>
       </c>
+      <c r="G51" s="6" t="n"/>
+      <c r="H51" s="6" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Law with English Language Studies</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="6" t="inlineStr">
         <is>
           <t>DEG-000051</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>English Studies</t>
         </is>
       </c>
-      <c r="E52" t="n">
+      <c r="E52" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F52" s="6" t="inlineStr">
         <is>
           <t>Combines law with advanced study of English linguistics and usage. Builds strong written and verbal reasoning. Prepares for careers in law, media, publishing, or public administration.</t>
         </is>
       </c>
+      <c r="G52" s="6" t="n"/>
+      <c r="H52" s="6" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Law with English</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>DEG-000052</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="E53" t="n">
+      <c r="E53" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <t>Combines law with English language and literature studies. Strengthens critical thinking, analysis, and communication. Prepares for careers in law, publishing, education, or media industries.</t>
         </is>
       </c>
+      <c r="G53" s="6" t="n"/>
+      <c r="H53" s="6" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Law with Classical Studies</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>DEG-000053</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>Classical Studies</t>
         </is>
       </c>
-      <c r="E54" t="n">
+      <c r="E54" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F54" s="6" t="inlineStr">
         <is>
           <t>Integrates law with ancient Greek and Roman civilizations. Develops analytical and historical interpretation skills. Prepares for careers in law, academia, heritage, or cultural policy sectors.</t>
         </is>
       </c>
+      <c r="G54" s="6" t="n"/>
+      <c r="H54" s="6" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Law with Criminology</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>DEG-000054</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>Criminology</t>
         </is>
       </c>
-      <c r="E55" t="n">
+      <c r="E55" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <t>Combines law with the study of crime, justice, and society. Develops understanding of criminal behavior and legal responses. Leads to careers in policing, legal practice, or criminal justice policy.</t>
         </is>
       </c>
+      <c r="G55" s="6" t="n"/>
+      <c r="H55" s="6" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Forestry Transfer</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="6" t="inlineStr">
         <is>
           <t>DEG-000055</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>Forestry (Transfer Program)</t>
         </is>
       </c>
-      <c r="E56" t="n">
+      <c r="E56" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F56" s="6" t="inlineStr">
         <is>
           <t>Provides foundational forestry education for academic transfer pathways. Develops basic ecological and scientific skills. Prepares students for advanced forestry studies. Strengthens academic readiness. Supports progression into specialized forestry degrees.</t>
         </is>
       </c>
+      <c r="G56" s="6" t="n"/>
+      <c r="H56" s="6" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Language and Literature Education</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>DEG-000056</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>Education &amp; Language</t>
         </is>
       </c>
-      <c r="E57" t="n">
+      <c r="E57" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F57" s="6" t="inlineStr">
         <is>
           <t>Focuses on teaching languages and literature. Builds pedagogy and communication skills. Graduates work as language teachers.</t>
         </is>
       </c>
+      <c r="G57" s="6" t="n"/>
+      <c r="H57" s="6" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Mathematics with Education</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="6" t="inlineStr">
         <is>
           <t>DEG-000057</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="6" t="inlineStr">
         <is>
           <t>Mathematics Education</t>
         </is>
       </c>
-      <c r="E58" t="n">
+      <c r="E58" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F58" s="6" t="inlineStr">
         <is>
           <t>Focuses on mathematics teaching and learning methods. Builds pedagogical skills. Graduates work in schools or education roles.</t>
         </is>
       </c>
+      <c r="G58" s="6" t="n"/>
+      <c r="H58" s="6" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Italian and Persian</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>DEG-000058</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>Language Studies</t>
         </is>
       </c>
-      <c r="E59" t="n">
+      <c r="E59" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="F59" s="6" t="inlineStr">
         <is>
           <t>Combines Italian and Persian languages. Builds intercultural communication skills. Graduates work in translation and diplomacy.</t>
         </is>
       </c>
+      <c r="G59" s="6" t="n"/>
+      <c r="H59" s="6" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="6" t="inlineStr">
         <is>
           <t>Bachelor of Medical Studies and Doctor of Medicine</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="6" t="inlineStr">
         <is>
           <t>DEG-000059</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D60" s="6" t="inlineStr">
         <is>
           <t>Medical Pathway</t>
         </is>
       </c>
-      <c r="E60" t="n">
+      <c r="E60" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="F60" s="6" t="inlineStr">
         <is>
           <t>Integrated medical training program. Builds clinical and scientific expertise. Graduates become licensed medical practitioners.</t>
         </is>
       </c>
+      <c r="G60" s="6" t="n"/>
+      <c r="H60" s="6" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="6" t="inlineStr">
         <is>
           <t>Bachelor of History Teaching</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="6" t="inlineStr">
         <is>
           <t>DEG-000060</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="6" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61" s="6" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E61" t="n">
+      <c r="E61" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="F61" s="6" t="inlineStr">
         <is>
           <t>Studies methods of teaching history. Develops pedagogical skills. Focuses on classroom instruction. Graduates work as educators.</t>
         </is>
       </c>
+      <c r="G61" s="6" t="n"/>
+      <c r="H61" s="6" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="6" t="inlineStr">
         <is>
           <t>PhD in Fluids Engineering</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="6" t="inlineStr">
         <is>
           <t>DEG-000061</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62" s="6" t="inlineStr">
         <is>
           <t>Mechanical Engineering</t>
         </is>
       </c>
-      <c r="E62" t="n">
+      <c r="E62" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="F62" s="6" t="inlineStr">
         <is>
           <t>Studies fluid flow and engineering system design. Develops expertise in computational modeling and experimental research. Focuses on industrial and energy applications. Graduates work in research, aerospace, and engineering firms.</t>
         </is>
       </c>
+      <c r="G62" s="6" t="n"/>
+      <c r="H62" s="6" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="6" t="inlineStr">
         <is>
           <t>PhD in Food and Biochemical Technology</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="6" t="inlineStr">
         <is>
           <t>DEG-000062</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D63" s="6" t="inlineStr">
         <is>
           <t>Food Science</t>
         </is>
       </c>
-      <c r="E63" t="n">
+      <c r="E63" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F63" s="6" t="inlineStr">
         <is>
           <t>Combines food science with biochemical technologies. Develops expertise in food processing and biochemical research. Focuses on improving food quality and innovation. Graduates work in academia, biotechnology, and food industries.</t>
         </is>
       </c>
+      <c r="G63" s="6" t="n"/>
+      <c r="H63" s="6" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="6" t="inlineStr">
         <is>
           <t>PhD in Food Systems</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="6" t="inlineStr">
         <is>
           <t>DEG-000063</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="6" t="inlineStr">
         <is>
           <t>Food Systems</t>
         </is>
       </c>
-      <c r="E64" t="n">
+      <c r="E64" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F64" s="6" t="inlineStr">
         <is>
           <t>Explores food production, distribution, and consumption systems. Develops interdisciplinary research and policy skills. Focuses on sustainability and resilience. Graduates work in academia, government, and nonprofit organizations.</t>
         </is>
       </c>
+      <c r="G64" s="6" t="n"/>
+      <c r="H64" s="6" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="6" t="inlineStr">
         <is>
           <t>PhD in Gender Studies</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B65" s="6" t="inlineStr">
         <is>
           <t>DEG-000064</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65" s="6" t="inlineStr">
         <is>
           <t>Gender Studies</t>
         </is>
       </c>
-      <c r="E65" t="n">
+      <c r="E65" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F65" s="6" t="inlineStr">
         <is>
           <t>Explores gender through social, political, and cultural research. Develops critical thinking and interdisciplinary research skills. Focuses on identity and equality. Graduates work in academia, policy, and community organizations.</t>
         </is>
       </c>
+      <c r="G65" s="6" t="n"/>
+      <c r="H65" s="6" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="6" t="inlineStr">
         <is>
           <t>PhD in Geodesy and Geoinformatics</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="6" t="inlineStr">
         <is>
           <t>DEG-000065</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D66" s="6" t="inlineStr">
         <is>
           <t>Geospatial Science</t>
         </is>
       </c>
-      <c r="E66" t="n">
+      <c r="E66" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F66" s="6" t="inlineStr">
         <is>
           <t>Combines geodesy with digital geographic information systems. Develops expertise in spatial analysis and geospatial technologies. Focuses on Earth measurement and mapping. Graduates work in academia, surveying, and GIS industries.</t>
         </is>
       </c>
+      <c r="G66" s="6" t="n"/>
+      <c r="H66" s="6" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="6" t="inlineStr">
         <is>
           <t>PhD in Geography and Earth Science</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B67" s="6" t="inlineStr">
         <is>
           <t>DEG-000066</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D67" s="6" t="inlineStr">
         <is>
           <t>Earth Science</t>
         </is>
       </c>
-      <c r="E67" t="n">
+      <c r="E67" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="F67" s="6" t="inlineStr">
         <is>
           <t>Combines geography with Earth science research. Develops expertise in environmental systems and geospatial analysis. Focuses on understanding Earth's processes. Graduates work in academia, environmental consulting, and government.</t>
         </is>
       </c>
+      <c r="G67" s="6" t="n"/>
+      <c r="H67" s="6" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="6" t="inlineStr">
         <is>
           <t>PhD in Geometry and Topology</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B68" s="6" t="inlineStr">
         <is>
           <t>DEG-000067</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr">
+      <c r="D68" s="6" t="inlineStr">
         <is>
           <t>Mathematics</t>
         </is>
       </c>
-      <c r="E68" t="n">
+      <c r="E68" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="F68" s="6" t="inlineStr">
         <is>
           <t>Studies the properties and structures of geometric spaces. Develops expertise in abstract mathematics and theoretical research. Focuses on advanced mathematical concepts. Graduates work in academia, research, and higher education.</t>
         </is>
       </c>
+      <c r="G68" s="6" t="n"/>
+      <c r="H68" s="6" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="6" t="inlineStr">
         <is>
           <t>PhD in Geospatial Analytics</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="6" t="inlineStr">
         <is>
           <t>DEG-000068</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D69" s="6" t="inlineStr">
         <is>
           <t>Data Science</t>
         </is>
       </c>
-      <c r="E69" t="n">
+      <c r="E69" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F69" s="6" t="inlineStr">
         <is>
           <t>Studies advanced analysis of geographic and spatial data. Develops expertise in GIS, machine learning, and predictive modeling. Focuses on spatial decision-making. Graduates work in academia, government, and technology industries.</t>
         </is>
       </c>
+      <c r="G69" s="6" t="n"/>
+      <c r="H69" s="6" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="6" t="inlineStr">
         <is>
           <t>PhD in Grain Science</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B70" s="6" t="inlineStr">
         <is>
           <t>DEG-000069</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C70" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D70" s="6" t="inlineStr">
         <is>
           <t>Agricultural Science</t>
         </is>
       </c>
-      <c r="E70" t="n">
+      <c r="E70" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="F70" s="6" t="inlineStr">
         <is>
           <t>Studies grain production, processing, and quality. Develops expertise in cereal chemistry and agricultural research. Focuses on food quality and sustainable production. Graduates work in academia, agriculture, and food industries.</t>
         </is>
       </c>
+      <c r="G70" s="6" t="n"/>
+      <c r="H70" s="6" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
+      <c r="A71" s="6" t="inlineStr">
         <is>
           <t>PhD in Health Economics and Policy</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B71" s="6" t="inlineStr">
         <is>
           <t>DEG-000070</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C71" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr">
+      <c r="D71" s="6" t="inlineStr">
         <is>
           <t>Health Economics</t>
         </is>
       </c>
-      <c r="E71" t="n">
+      <c r="E71" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="F71" s="6" t="inlineStr">
         <is>
           <t>Integrates economic analysis with healthcare policy research. Develops expertise in health financing and policy evaluation. Focuses on improving health systems. Graduates work in academia, government, and healthcare organizations.</t>
         </is>
       </c>
+      <c r="G71" s="6" t="n"/>
+      <c r="H71" s="6" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
+      <c r="A72" s="6" t="inlineStr">
         <is>
           <t>PhD in Hispanic Studies and Comparative Literature</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B72" s="6" t="inlineStr">
         <is>
           <t>DEG-000071</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C72" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D72" s="6" t="inlineStr">
         <is>
           <t>Literature</t>
         </is>
       </c>
-      <c r="E72" t="n">
+      <c r="E72" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F72" s="6" t="inlineStr">
         <is>
           <t>Combines Hispanic studies with comparative literary research. Develops expertise in literary analysis and cross-cultural interpretation. Focuses on global literary traditions. Graduates work in academia, publishing, and education.</t>
         </is>
       </c>
+      <c r="G72" s="6" t="n"/>
+      <c r="H72" s="6" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
+      <c r="A73" s="6" t="inlineStr">
         <is>
           <t>PhD in History of Art and Archaeology</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B73" s="6" t="inlineStr">
         <is>
           <t>DEG-000072</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C73" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D73" s="6" t="inlineStr">
         <is>
           <t>Art History</t>
         </is>
       </c>
-      <c r="E73" t="n">
+      <c r="E73" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F73" s="6" t="inlineStr">
         <is>
           <t>Combines art history with archaeological research. Develops expertise in material culture and historical interpretation. Focuses on ancient and historical artifacts. Graduates work in academia, museums, and heritage organizations.</t>
         </is>
       </c>
+      <c r="G73" s="6" t="n"/>
+      <c r="H73" s="6" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="A74" s="6" t="inlineStr">
         <is>
           <t>PhD in Laser, Photonics and Vision</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B74" s="6" t="inlineStr">
         <is>
           <t>DEG-000073</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C74" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D74" s="6" t="inlineStr">
         <is>
           <t>Physics</t>
         </is>
       </c>
-      <c r="E74" t="n">
+      <c r="E74" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="F74" s="6" t="inlineStr">
         <is>
           <t>Studies laser systems, photonics, and optical vision technologies. Develops expertise in optics, imaging, and applied physics. Focuses on light-based technologies. Graduates work in academia, research labs, and optical industries.</t>
         </is>
       </c>
+      <c r="G74" s="6" t="n"/>
+      <c r="H74" s="6" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="6" t="inlineStr">
         <is>
           <t>PhD in Latin American Cultural Studies</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B75" s="6" t="inlineStr">
         <is>
           <t>DEG-000074</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D75" s="6" t="inlineStr">
         <is>
           <t>Cultural Studies</t>
         </is>
       </c>
-      <c r="E75" t="n">
+      <c r="E75" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F75" s="6" t="inlineStr">
         <is>
           <t>Explores cultural production, identity, and history in Latin America. Develops expertise in literary and cultural theory. Focuses on regional cultural expression. Graduates work in academia, publishing, and cultural organizations.</t>
         </is>
       </c>
+      <c r="G75" s="6" t="n"/>
+      <c r="H75" s="6" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" s="6" t="inlineStr">
         <is>
           <t>PhD in Leadership and Policy Studies in Education</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="6" t="inlineStr">
         <is>
           <t>DEG-000075</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C76" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D76" s="6" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="E76" t="n">
+      <c r="E76" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F76" s="6" t="inlineStr">
         <is>
           <t>Examines leadership and policy in educational systems. Develops expertise in administration, policy analysis, and school leadership. Focuses on educational improvement. Graduates work in academia, schools, and government agencies.</t>
         </is>
       </c>
+      <c r="G76" s="6" t="n"/>
+      <c r="H76" s="6" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
+      <c r="A77" s="6" t="inlineStr">
         <is>
           <t>PhD in Management Finance</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B77" s="6" t="inlineStr">
         <is>
           <t>DEG-000076</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C77" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D77" s="6" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="E77" t="n">
+      <c r="E77" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F77" t="inlineStr">
+      <c r="F77" s="6" t="inlineStr">
         <is>
           <t>Integrates financial management with organizational strategy. Develops expertise in corporate finance, investment, and risk management. Focuses on financial decision-making. Graduates work in finance, corporations, and consulting.</t>
         </is>
       </c>
+      <c r="G77" s="6" t="n"/>
+      <c r="H77" s="6" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
+      <c r="A78" s="6" t="inlineStr">
         <is>
           <t>PhD in Marine Engine Engineering</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="B78" s="6" t="inlineStr">
         <is>
           <t>DEG-000077</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C78" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="D78" s="6" t="inlineStr">
         <is>
           <t>Marine Engineering</t>
         </is>
       </c>
-      <c r="E78" t="n">
+      <c r="E78" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F78" t="inlineStr">
+      <c r="F78" s="6" t="inlineStr">
         <is>
           <t>Focuses on design and maintenance of marine propulsion systems. Develops expertise in mechanical and marine systems engineering. Focuses on ship engine performance. Graduates work in shipping, engineering, and maritime industries.</t>
         </is>
       </c>
+      <c r="G78" s="6" t="n"/>
+      <c r="H78" s="6" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
+      <c r="A79" s="6" t="inlineStr">
         <is>
           <t>PhD in Marketing and Entrepreneurship</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B79" s="6" t="inlineStr">
         <is>
           <t>DEG-000078</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C79" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D79" s="6" t="inlineStr">
         <is>
           <t>Entrepreneurship</t>
         </is>
       </c>
-      <c r="E79" t="n">
+      <c r="E79" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F79" t="inlineStr">
+      <c r="F79" s="6" t="inlineStr">
         <is>
           <t>Studies marketing strategies for new ventures and startups. Develops expertise in innovation, branding, and business development. Focuses on entrepreneurial growth. Graduates work in startups, consulting, and business development.</t>
         </is>
       </c>
+      <c r="G79" s="6" t="n"/>
+      <c r="H79" s="6" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
+      <c r="A80" s="6" t="inlineStr">
         <is>
           <t>PhD in Phonetics and Phonology</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B80" s="6" t="inlineStr">
         <is>
           <t>DEG-000079</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C80" s="6" t="inlineStr">
         <is>
           <t>PhD</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr">
+      <c r="D80" s="6" t="inlineStr">
         <is>
           <t>Linguistics</t>
         </is>
       </c>
-      <c r="E80" t="n">
+      <c r="E80" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F80" t="inlineStr">
+      <c r="F80" s="6" t="inlineStr">
         <is>
           <t>Combines speech sound analysis with language sound systems. Develops expertise in linguistic theory and speech research. Focuses on sound structure and communication. Graduates work in academia, linguistics, and speech technology.</t>
         </is>
       </c>
+      <c r="G80" s="6" t="n"/>
+      <c r="H80" s="6" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
+      <c r="A81" s="6" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Nursing and Allied Health</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B81" s="6" t="inlineStr">
         <is>
           <t>DEG-000080</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C81" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D81" s="6" t="inlineStr">
         <is>
           <t>Nursing and Allied Health</t>
         </is>
       </c>
-      <c r="E81" t="n">
-        <v>2</v>
-      </c>
-      <c r="F81" t="inlineStr">
+      <c r="E81" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F81" s="6" t="inlineStr">
         <is>
           <t>Studies basic nursing and healthcare support. Develops clinical and patient care skills. Focuses on healthcare services. Prepares graduates for healthcare support roles.</t>
         </is>
       </c>
+      <c r="G81" s="6" t="n"/>
+      <c r="H81" s="6" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
+      <c r="A82" s="6" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Medical Assistant</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B82" s="6" t="inlineStr">
         <is>
           <t>DEG-000081</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C82" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr">
+      <c r="D82" s="6" t="inlineStr">
         <is>
           <t>Medical Assistance</t>
         </is>
       </c>
-      <c r="E82" t="n">
-        <v>2</v>
-      </c>
-      <c r="F82" t="inlineStr">
+      <c r="E82" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F82" s="6" t="inlineStr">
         <is>
           <t>Studies clinical and administrative healthcare support. Develops patient care skills. Focuses on medical office practice. Prepares graduates for healthcare support roles.</t>
         </is>
       </c>
+      <c r="G82" s="6" t="n"/>
+      <c r="H82" s="6" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
+      <c r="A83" s="6" t="inlineStr">
         <is>
           <t>Associate of Science in Radiography</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="B83" s="6" t="inlineStr">
         <is>
           <t>DEG-000082</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C83" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
+      <c r="D83" s="6" t="inlineStr">
         <is>
           <t>Radiography</t>
         </is>
       </c>
-      <c r="E83" t="n">
-        <v>2</v>
-      </c>
-      <c r="F83" t="inlineStr">
+      <c r="E83" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F83" s="6" t="inlineStr">
         <is>
           <t>Studies medical imaging and radiographic techniques. Develops imaging, patient care, and technical skills. Focuses on diagnostic imaging procedures. Graduates work in hospitals and medical imaging departments.</t>
         </is>
       </c>
+      <c r="G83" s="6" t="n"/>
+      <c r="H83" s="6" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
+      <c r="A84" s="6" t="inlineStr">
         <is>
           <t>Associate of Arts in Marketing</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B84" s="6" t="inlineStr">
         <is>
           <t>DEG-000083</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C84" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="D84" s="6" t="inlineStr">
         <is>
           <t>Marketing</t>
         </is>
       </c>
-      <c r="E84" t="n">
-        <v>2</v>
-      </c>
-      <c r="F84" t="inlineStr">
+      <c r="E84" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F84" s="6" t="inlineStr">
         <is>
           <t>Studies marketing strategies and consumer behavior. Develops communication, analytical, and promotional skills. Focuses on branding, advertising, and market research. Graduates work in marketing, sales, and retail.</t>
         </is>
       </c>
+      <c r="G84" s="6" t="n"/>
+      <c r="H84" s="6" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
+      <c r="A85" s="6" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Dental Hygiene</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B85" s="6" t="inlineStr">
         <is>
           <t>DEG-000084</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C85" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D85" s="6" t="inlineStr">
         <is>
           <t>Dental Hygiene</t>
         </is>
       </c>
-      <c r="E85" t="n">
-        <v>2</v>
-      </c>
-      <c r="F85" t="inlineStr">
+      <c r="E85" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" s="6" t="inlineStr">
         <is>
           <t>Studies preventive dental care and oral health. Develops clinical, patient care, and communication skills. Focuses on dental hygiene procedures and education. Graduates work in dental clinics and healthcare facilities.</t>
         </is>
       </c>
+      <c r="G85" s="6" t="n"/>
+      <c r="H85" s="6" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
+      <c r="A86" s="6" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Radiography</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B86" s="6" t="inlineStr">
         <is>
           <t>DEG-000085</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C86" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D86" s="6" t="inlineStr">
         <is>
           <t>Radiography</t>
         </is>
       </c>
-      <c r="E86" t="n">
-        <v>2</v>
-      </c>
-      <c r="F86" t="inlineStr">
+      <c r="E86" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F86" s="6" t="inlineStr">
         <is>
           <t>Studies diagnostic imaging and radiographic procedures. Develops imaging, patient care, and technical skills. Focuses on producing medical images for diagnosis. Graduates work in hospitals and diagnostic imaging centers.</t>
         </is>
       </c>
+      <c r="G86" s="6" t="n"/>
+      <c r="H86" s="6" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
+      <c r="A87" s="6" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Diagnostic Medical Sonography</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B87" s="6" t="inlineStr">
         <is>
           <t>DEG-000086</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C87" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D87" s="6" t="inlineStr">
         <is>
           <t>Diagnostic Medical Sonography</t>
         </is>
       </c>
-      <c r="E87" t="n">
-        <v>2</v>
-      </c>
-      <c r="F87" t="inlineStr">
+      <c r="E87" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F87" s="6" t="inlineStr">
         <is>
           <t>Studies ultrasound imaging and patient care. Develops diagnostic imaging, technical, and clinical skills. Focuses on safe and accurate medical sonography. Prepares graduates for careers as diagnostic medical sonographers.</t>
         </is>
       </c>
+      <c r="G87" s="6" t="n"/>
+      <c r="H87" s="6" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr">
+      <c r="A88" s="6" t="inlineStr">
         <is>
           <t>Associate of Science in Music Production</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B88" s="6" t="inlineStr">
         <is>
           <t>DEG-000087</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="C88" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="D88" s="6" t="inlineStr">
         <is>
           <t>Music Production</t>
         </is>
       </c>
-      <c r="E88" t="n">
-        <v>2</v>
-      </c>
-      <c r="F88" t="inlineStr">
+      <c r="E88" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F88" s="6" t="inlineStr">
         <is>
           <t>Studies audio recording, music technology, and production. Develops recording, editing, and sound design skills. Focuses on creating professional music productions. Graduates work in recording studios and media production.</t>
         </is>
       </c>
+      <c r="G88" s="6" t="n"/>
+      <c r="H88" s="6" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr">
+      <c r="A89" s="6" t="inlineStr">
         <is>
           <t>Associate of Applied Science</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B89" s="6" t="inlineStr">
         <is>
           <t>DEG-000088</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C89" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="D89" s="6" t="inlineStr">
         <is>
           <t>Applied Science</t>
         </is>
       </c>
-      <c r="E89" t="n">
-        <v>2</v>
-      </c>
-      <c r="F89" t="inlineStr">
+      <c r="E89" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F89" s="6" t="inlineStr">
         <is>
           <t>Studies practical scientific and technical applications. Develops laboratory, technical, and problem-solving skills. Focuses on career-ready scientific knowledge. Graduates work in technical, healthcare, and industrial roles.</t>
         </is>
       </c>
+      <c r="G89" s="6" t="n"/>
+      <c r="H89" s="6" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr">
+      <c r="A90" s="6" t="inlineStr">
         <is>
           <t>Associate of Science in Nursing</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B90" s="6" t="inlineStr">
         <is>
           <t>DEG-000089</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C90" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr">
+      <c r="D90" s="6" t="inlineStr">
         <is>
           <t>Nursing</t>
         </is>
       </c>
-      <c r="E90" t="n">
-        <v>2</v>
-      </c>
-      <c r="F90" t="inlineStr">
+      <c r="E90" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F90" s="6" t="inlineStr">
         <is>
           <t>Studies nursing science and patient-centered care. Develops clinical, communication, and healthcare skills. Focuses on safe nursing practice and health promotion. Graduates work in hospitals, clinics, and healthcare facilities.</t>
         </is>
       </c>
+      <c r="G90" s="6" t="n"/>
+      <c r="H90" s="6" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr">
+      <c r="A91" s="6" t="inlineStr">
         <is>
           <t>Associate of Arts</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B91" s="6" t="inlineStr">
         <is>
           <t>DEG-000090</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C91" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr">
+      <c r="D91" s="6" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="E91" t="n">
-        <v>2</v>
-      </c>
-      <c r="F91" t="inlineStr">
+      <c r="E91" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F91" s="6" t="inlineStr">
         <is>
           <t>Studies humanities, social sciences, and communication. Develops critical thinking, writing, and analytical skills. Focuses on broad academic preparation. Graduates continue higher education or enter diverse professional fields.</t>
         </is>
       </c>
+      <c r="G91" s="6" t="n"/>
+      <c r="H91" s="6" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
+      <c r="A92" s="6" t="inlineStr">
         <is>
           <t>Associate of Arts Degree</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
+      <c r="B92" s="6" t="inlineStr">
         <is>
           <t>DEG-000091</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
+      <c r="C92" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr">
+      <c r="D92" s="6" t="inlineStr">
         <is>
           <t>Liberal Arts</t>
         </is>
       </c>
-      <c r="E92" t="n">
-        <v>2</v>
-      </c>
-      <c r="F92" t="inlineStr">
+      <c r="E92" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F92" s="6" t="inlineStr">
         <is>
           <t>Studies a broad range of humanities and social sciences. Develops communication, research, and critical thinking skills. Focuses on transferable academic knowledge. Graduates continue higher education or pursue entry-level careers.</t>
         </is>
       </c>
+      <c r="G92" s="6" t="n"/>
+      <c r="H92" s="6" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr">
+      <c r="A93" s="6" t="inlineStr">
         <is>
           <t>Associate of Nursing</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B93" s="6" t="inlineStr">
         <is>
           <t>DEG-000092</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C93" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr">
+      <c r="D93" s="6" t="inlineStr">
         <is>
           <t>Nursing</t>
         </is>
       </c>
-      <c r="E93" t="n">
-        <v>2</v>
-      </c>
-      <c r="F93" t="inlineStr">
+      <c r="E93" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F93" s="6" t="inlineStr">
         <is>
           <t>Studies patient care and foundational nursing practice. Develops clinical, communication, and healthcare skills. Focuses on evidence-based nursing and patient safety. Graduates work in hospitals, clinics, and healthcare facilities.</t>
         </is>
       </c>
+      <c r="G93" s="6" t="n"/>
+      <c r="H93" s="6" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr">
+      <c r="A94" s="6" t="inlineStr">
         <is>
           <t>Associate of Science in Business</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B94" s="6" t="inlineStr">
         <is>
           <t>DEG-000093</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
+      <c r="C94" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr">
+      <c r="D94" s="6" t="inlineStr">
         <is>
           <t>Business</t>
         </is>
       </c>
-      <c r="E94" t="n">
-        <v>2</v>
-      </c>
-      <c r="F94" t="inlineStr">
+      <c r="E94" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F94" s="6" t="inlineStr">
         <is>
           <t>Studies core business principles and organizational practices. Develops communication, management, and analytical skills. Focuses on finance, marketing, and operations. Graduates work in business support, retail, and administration.</t>
         </is>
       </c>
+      <c r="G94" s="6" t="n"/>
+      <c r="H94" s="6" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr">
+      <c r="A95" s="6" t="inlineStr">
         <is>
           <t>Associate of Science</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="B95" s="6" t="inlineStr">
         <is>
           <t>DEG-000094</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C95" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr">
+      <c r="D95" s="6" t="inlineStr">
         <is>
           <t>Science</t>
         </is>
       </c>
-      <c r="E95" t="n">
-        <v>2</v>
-      </c>
-      <c r="F95" t="inlineStr">
+      <c r="E95" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F95" s="6" t="inlineStr">
         <is>
           <t>Studies foundational scientific concepts and methods. Develops laboratory, analytical, and problem-solving skills. Focuses on biology, chemistry, and scientific inquiry. Graduates continue science studies or work in technical fields.</t>
         </is>
       </c>
+      <c r="G95" s="6" t="n"/>
+      <c r="H95" s="6" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
+      <c r="A96" s="6" t="inlineStr">
         <is>
           <t>Associate of Science in Business Administration</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B96" s="6" t="inlineStr">
         <is>
           <t>DEG-000095</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C96" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr">
+      <c r="D96" s="6" t="inlineStr">
         <is>
           <t>Business Administration</t>
         </is>
       </c>
-      <c r="E96" t="n">
-        <v>2</v>
-      </c>
-      <c r="F96" t="inlineStr">
+      <c r="E96" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F96" s="6" t="inlineStr">
         <is>
           <t>Studies business operations and management fundamentals. Develops organizational, communication, and leadership skills. Focuses on business strategy and workplace effectiveness. Graduates work in administration, sales, and operations.</t>
         </is>
       </c>
+      <c r="G96" s="6" t="n"/>
+      <c r="H96" s="6" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
+      <c r="A97" s="6" t="inlineStr">
         <is>
           <t>Associate of Science in Biology and Ecology</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="B97" s="6" t="inlineStr">
         <is>
           <t>DEG-000096</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
+      <c r="C97" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr">
+      <c r="D97" s="6" t="inlineStr">
         <is>
           <t>Biology and Ecology</t>
         </is>
       </c>
-      <c r="E97" t="n">
-        <v>2</v>
-      </c>
-      <c r="F97" t="inlineStr">
+      <c r="E97" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F97" s="6" t="inlineStr">
         <is>
           <t>Studies biological systems and ecological processes. Develops laboratory, fieldwork, and analytical skills. Focuses on ecosystems, biodiversity, and environmental science. Graduates work in environmental organizations and laboratories.</t>
         </is>
       </c>
+      <c r="G97" s="6" t="n"/>
+      <c r="H97" s="6" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
+      <c r="A98" s="6" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Accounting</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
+      <c r="B98" s="6" t="inlineStr">
         <is>
           <t>DEG-000097</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
+      <c r="C98" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr">
+      <c r="D98" s="6" t="inlineStr">
         <is>
           <t>Accounting</t>
         </is>
       </c>
-      <c r="E98" t="n">
-        <v>2</v>
-      </c>
-      <c r="F98" t="inlineStr">
+      <c r="E98" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F98" s="6" t="inlineStr">
         <is>
           <t>Studies accounting principles and financial reporting. Develops bookkeeping, financial analysis, and accounting software skills. Focuses on business finance and compliance. Graduates work in accounting, bookkeeping, and finance support.</t>
         </is>
       </c>
+      <c r="G98" s="6" t="n"/>
+      <c r="H98" s="6" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr">
+      <c r="A99" s="6" t="inlineStr">
         <is>
           <t>Associate of Applied Science in Hospitality Management</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="B99" s="6" t="inlineStr">
         <is>
           <t>DEG-000098</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C99" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr">
+      <c r="D99" s="6" t="inlineStr">
         <is>
           <t>Hospitality Management</t>
         </is>
       </c>
-      <c r="E99" t="n">
-        <v>2</v>
-      </c>
-      <c r="F99" t="inlineStr">
+      <c r="E99" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F99" s="6" t="inlineStr">
         <is>
           <t>Studies hospitality operations and customer service management. Develops leadership, communication, and operational skills. Focuses on hotels, tourism, and guest satisfaction. Graduates work in hospitality, tourism, and hotel management.</t>
         </is>
       </c>
+      <c r="G99" s="6" t="n"/>
+      <c r="H99" s="6" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr">
+      <c r="A100" s="6" t="inlineStr">
         <is>
           <t>Associate of Science in Computer Science</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
+      <c r="B100" s="6" t="inlineStr">
         <is>
           <t>DEG-000099</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
+      <c r="C100" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr">
+      <c r="D100" s="6" t="inlineStr">
         <is>
           <t>Computer Science</t>
         </is>
       </c>
-      <c r="E100" t="n">
-        <v>2</v>
-      </c>
-      <c r="F100" t="inlineStr">
+      <c r="E100" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F100" s="6" t="inlineStr">
         <is>
           <t>Studies computing principles and software development. Develops programming, analytical, and technical problem-solving skills. Focuses on algorithms, databases, and computer systems. Graduates work in IT support and software development.</t>
         </is>
       </c>
+      <c r="G100" s="6" t="n"/>
+      <c r="H100" s="6" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
+      <c r="A101" s="6" t="inlineStr">
         <is>
           <t>Associate of Arts in Business Administration</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
+      <c r="B101" s="6" t="inlineStr">
         <is>
           <t>DEG-000100</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
+      <c r="C101" s="6" t="inlineStr">
         <is>
           <t>Associate</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr">
+      <c r="D101" s="6" t="inlineStr">
         <is>
           <t>Business Administration</t>
         </is>
       </c>
-      <c r="E101" t="n">
-        <v>2</v>
-      </c>
-      <c r="F101" t="inlineStr">
+      <c r="E101" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F101" s="6" t="inlineStr">
         <is>
           <t>Studies business operations and organizational management. Develops leadership, communication, and administrative skills. Focuses on finance, marketing, and business practices. Graduates work in administration, retail, and business support.</t>
         </is>
       </c>
+      <c r="G101" s="6" t="n"/>
+      <c r="H101" s="6" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1" password="DB2D"/>

</xml_diff>